<commit_message>
scan: seg4 2026-10-23 20:32 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq5_2026-10-22.xlsx
@@ -4608,21 +4608,21 @@
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>4924</v>
+        <v>4542</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>欣厚-KY</t>
+          <t>科嶠</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>453.5993382542297</v>
+        <v>454.9208084580185</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>19.15</v>
+        <v>345</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>60.02497464158744</v>
+        <v>52.02037519710391</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>35.68442794600203</v>
+        <v>31.18402030353885</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.6708265725262842</v>
+        <v>1.180801934696807</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.1625535905581788</v>
+        <v>0.5544916636013539</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>4571</v>
+        <v>4924</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>鈞興-KY</t>
+          <t>欣厚-KY</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>449.7242502724685</v>
+        <v>453.5993382542297</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>158.5</v>
+        <v>19.15</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>55.46918353695793</v>
+        <v>60.02497464158744</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.24548215306085</v>
+        <v>35.68442794600203</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.6460041308695501</v>
+        <v>0.6708265725262842</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.7925144962944661</v>
+        <v>0.1625535905581788</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>5344</v>
+        <v>4571</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>立衛</t>
+          <t>鈞興-KY</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>448.7307920607385</v>
+        <v>449.7242502724685</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>13.65</v>
+        <v>158.5</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>49.61056871944271</v>
+        <v>55.46918353695793</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>29.06409280999027</v>
+        <v>14.24548215306085</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.1924478965139438</v>
+        <v>0.6460041308695501</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.01490187001014669</v>
+        <v>0.7925144962944661</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>4915</v>
+        <v>5344</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>致伸</t>
+          <t>立衛</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>447.1863521922414</v>
+        <v>448.7307920607385</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>62</v>
+        <v>13.65</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>43.4057325521774</v>
+        <v>49.61056871944271</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>20.97532757266605</v>
+        <v>29.06409280999027</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.339903640251592</v>
+        <v>0.1924478965139438</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.3008378255459638</v>
+        <v>-0.01490187001014669</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>4967</v>
+        <v>4915</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>十銓</t>
+          <t>致伸</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>445.0492209956828</v>
+        <v>447.1863521922414</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>250</v>
+        <v>62</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,16 +4845,16 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>35.80855122076545</v>
+        <v>43.4057325521774</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>17.1592585902746</v>
+        <v>20.97532757266605</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.6246090928836558</v>
+        <v>1.339903640251592</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-2.231573269097224</v>
+        <v>-0.3008378255459638</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
+          <t>avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>5244</v>
+        <v>4967</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>弘凱</t>
+          <t>十銓</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>444.2470702293381</v>
+        <v>445.0492209956828</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>36.4</v>
+        <v>250</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,16 +4898,16 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>49.06128084638738</v>
+        <v>35.80855122076545</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>16.54223330662872</v>
+        <v>17.1592585902746</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.3477868282759332</v>
+        <v>0.6246090928836558</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.2913614050573083</v>
+        <v>-2.231573269097224</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6155</v>
+        <v>5244</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>弘凱</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>440.1113795733072</v>
+        <v>444.2470702293381</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>69.5</v>
+        <v>36.4</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>56.30428730938871</v>
+        <v>49.06128084638738</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>26.8374818159345</v>
+        <v>16.54223330662872</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>1.392288391984023</v>
+        <v>0.3477868282759332</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.2875674543175464</v>
+        <v>-0.2913614050573083</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>4999</v>
+        <v>6155</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>鑫禾</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>434.6857687521248</v>
+        <v>440.1113795733072</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>17.3</v>
+        <v>69.5</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>31.85403101335631</v>
+        <v>56.30428730938871</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>37.7884122994969</v>
+        <v>26.8374818159345</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.918010049699698</v>
+        <v>1.392288391984023</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.01017590790040424</v>
+        <v>-0.2875674543175464</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6116</v>
+        <v>4999</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>彩晶</t>
+          <t>鑫禾</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>432.6029950513782</v>
+        <v>434.6857687521248</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>14.4</v>
+        <v>17.3</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>44.9675967026685</v>
+        <v>31.85403101335631</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>30.32974194865839</v>
+        <v>37.7884122994969</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.3184646564163551</v>
+        <v>0.918010049699698</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.1281383474927366</v>
+        <v>-0.01017590790040424</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>4935</v>
+        <v>6116</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>茂林-KY</t>
+          <t>彩晶</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>427.0369970972579</v>
+        <v>432.6029950513782</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>33.55</v>
+        <v>14.4</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.66570625985877</v>
+        <v>44.9675967026685</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>22.42465590057033</v>
+        <v>30.32974194865839</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>0.3145166128189087</v>
+        <v>0.3184646564163551</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.001360200883326113</v>
+        <v>-0.1281383474927366</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>5351</v>
+        <v>4935</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>鈺創</t>
+          <t>茂林-KY</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>425.0706277617496</v>
+        <v>427.0369970972579</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>100</v>
+        <v>33.55</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>40.42281237908083</v>
+        <v>49.66570625985877</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>13.54499920292864</v>
+        <v>22.42465590057033</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.6523495815408242</v>
+        <v>0.3145166128189087</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-1.185893966075786</v>
+        <v>0.001360200883326113</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>5522</v>
+        <v>5351</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>遠雄</t>
+          <t>鈺創</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>419.1509680386656</v>
+        <v>425.0706277617496</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>62.1</v>
+        <v>100</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>52.70391104792866</v>
+        <v>40.42281237908083</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>12.30888442507745</v>
+        <v>13.54499920292864</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.9233647726624306</v>
+        <v>0.6523495815408242</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.2038132078206641</v>
+        <v>-1.185893966075786</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>4971</v>
+        <v>5522</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>IET-KY</t>
+          <t>遠雄</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>416.7405722250556</v>
+        <v>419.1509680386656</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>450</v>
+        <v>62.1</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>34.87559538983402</v>
+        <v>52.70391104792866</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.96497700967682</v>
+        <v>12.30888442507745</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.6578222675025817</v>
+        <v>0.9233647726624306</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-13.24911078500627</v>
+        <v>0.2038132078206641</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, foreign_buy_3d, mfi_strong</t>
+          <t>avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>4991</v>
+        <v>4971</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>環宇-KY</t>
+          <t>IET-KY</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>413.8406231823269</v>
+        <v>416.7405722250556</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>415</v>
+        <v>450</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,49 +5322,49 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>39.09931715249833</v>
+        <v>34.87559538983402</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>11.58223382264858</v>
+        <v>16.96497700967682</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.6426868025653274</v>
+        <v>0.6578222675025817</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L92" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M92" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-8.233670897914932</v>
+        <v>-13.24911078500627</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6147</v>
+        <v>4991</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>頎邦</t>
+          <t>環宇-KY</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>411.2744933713344</v>
+        <v>413.8406231823269</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>203</v>
+        <v>415</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,49 +5375,49 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>46.62616352667133</v>
+        <v>39.09931715249833</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>20.74162651487287</v>
+        <v>11.58223382264858</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.4878336344862177</v>
+        <v>0.6426868025653274</v>
       </c>
       <c r="K93" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L93" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M93" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-3.566679099418293</v>
+        <v>-8.233670897914932</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, invest_trust_buy_2d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>4771</v>
+        <v>6147</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>望隼</t>
+          <t>頎邦</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>409.4972661636676</v>
+        <v>411.2744933713344</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>206.5</v>
+        <v>203</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>49.27639964223666</v>
+        <v>46.62616352667133</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.03993738986184</v>
+        <v>20.74162651487287</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.5821020311408892</v>
+        <v>0.4878336344862177</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.1706137507478546</v>
+        <v>-3.566679099418293</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, foreign_buy_3d, stronger_than_market</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>4755</v>
+        <v>4771</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>三福化</t>
+          <t>望隼</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>408.8057594870941</v>
+        <v>409.4972661636676</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>120</v>
+        <v>206.5</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.96259856797898</v>
+        <v>49.27639964223666</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>30.19699358240646</v>
+        <v>14.03993738986184</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.7298314301957985</v>
+        <v>0.5821020311408892</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.4364919034771391</v>
+        <v>-0.1706137507478546</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, foreign_buy_3d, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>4588</v>
+        <v>4755</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>玖鼎電力</t>
+          <t>三福化</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>407.3259486349922</v>
+        <v>408.8057594870941</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>55.4</v>
+        <v>120</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>51.47993810467231</v>
+        <v>47.96259856797898</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>24.67226665065835</v>
+        <v>30.19699358240646</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>1.07424450654123</v>
+        <v>0.7298314301957985</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.2672424729331937</v>
+        <v>-0.4364919034771391</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>4923</v>
+        <v>4588</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>力士</t>
+          <t>玖鼎電力</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>407.3230362459461</v>
+        <v>407.3259486349922</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>46.25</v>
+        <v>55.4</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.25653629714445</v>
+        <v>51.47993810467231</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>27.4078652412637</v>
+        <v>24.67226665065835</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.2688001915480837</v>
+        <v>1.07424450654123</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-1.767537340091067</v>
+        <v>-0.2672424729331937</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>4943</v>
+        <v>4923</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>康控-KY</t>
+          <t>力士</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>404.1887134156143</v>
+        <v>407.3230362459461</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>6.98</v>
+        <v>46.25</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>48.96009120091778</v>
+        <v>33.25653629714445</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.57627475015903</v>
+        <v>27.4078652412637</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.3522834717951072</v>
+        <v>0.2688001915480837</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.07548244276969551</v>
+        <v>-1.767537340091067</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6156</v>
+        <v>4943</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>松上</t>
+          <t>康控-KY</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>400.2799841675315</v>
+        <v>404.1887134156143</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>23.75</v>
+        <v>6.98</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>53.38968367484803</v>
+        <v>48.96009120091778</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>34.24851127541276</v>
+        <v>24.57627475015903</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.4439585338242862</v>
+        <v>0.3522834717951072</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.04489292534735034</v>
+        <v>0.07548244276969551</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>4931</v>
+        <v>6156</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>新盛力</t>
+          <t>松上</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>391.1618943845305</v>
+        <v>400.2799841675315</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>200</v>
+        <v>23.75</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>32.59205738302197</v>
+        <v>53.38968367484803</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>22.33610667961787</v>
+        <v>34.24851127541276</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.4706526780345856</v>
+        <v>0.4439585338242862</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-4.284881461155537</v>
+        <v>-0.04489292534735034</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>5258</v>
+        <v>4931</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>虹堡</t>
+          <t>新盛力</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>388.1162917329289</v>
+        <v>391.1618943845305</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>43.8</v>
+        <v>200</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>47.72205043711015</v>
+        <v>32.59205738302197</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>26.85301734232</v>
+        <v>22.33610667961787</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.7756948546847828</v>
+        <v>0.4706526780345856</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.3016156873566588</v>
+        <v>-4.284881461155537</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, foreign_buy_3d, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>5425</v>
+        <v>5258</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>台半</t>
+          <t>虹堡</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>387.0058066986779</v>
+        <v>388.1162917329289</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>88.8</v>
+        <v>43.8</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>41.2672045436275</v>
+        <v>47.72205043711015</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>18.25417875870735</v>
+        <v>26.85301734232</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.5628364826975915</v>
+        <v>0.7756948546847828</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-1.243661215438604</v>
+        <v>0.3016156873566588</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, foreign_buy_3d, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>5536</v>
+        <v>5425</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>聖暉*</t>
+          <t>台半</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>385.1555967426352</v>
+        <v>387.0058066986779</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>790</v>
+        <v>88.8</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>34.10721394905279</v>
+        <v>41.2672045436275</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>22.60116751255958</v>
+        <v>18.25417875870735</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.4155596742635219</v>
+        <v>0.5628364826975915</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-18.0524732425018</v>
+        <v>-1.243661215438604</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>5533</v>
+        <v>5536</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>皇鼎</t>
+          <t>聖暉*</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>382.9793271361722</v>
+        <v>385.1555967426352</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>13.9</v>
+        <v>790</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>48.02327140648779</v>
+        <v>34.10721394905279</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>16.54492496431556</v>
+        <v>22.60116751255958</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>1.41489103612369</v>
+        <v>0.4155596742635219</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.006273682245060475</v>
+        <v>-18.0524732425018</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
+          <t>avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>5489</v>
+        <v>5533</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>彩富</t>
+          <t>皇鼎</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>375.4686592806289</v>
+        <v>382.9793271361722</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>40.1</v>
+        <v>13.9</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>40.75018682499942</v>
+        <v>48.02327140648779</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>24.45809731486311</v>
+        <v>16.54492496431556</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.5398989861642104</v>
+        <v>1.41489103612369</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.1610759609064432</v>
+        <v>-0.006273682245060475</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>avoid_chase, stronger_than_market, kd_golden_cross, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>4912</v>
+        <v>5489</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>聯德控股-KY</t>
+          <t>彩富</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>372.2659009802676</v>
+        <v>375.4686592806289</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>95.40000000000001</v>
+        <v>40.1</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>40.00908294799905</v>
+        <v>40.75018682499942</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>19.24325210478369</v>
+        <v>24.45809731486311</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.3984613648528562</v>
+        <v>0.5398989861642104</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-1.395478721426864</v>
+        <v>-0.1610759609064432</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>5289</v>
+        <v>4912</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>宜鼎</t>
+          <t>聯德控股-KY</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>369.5531730137179</v>
+        <v>372.2659009802676</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>1065</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,49 +6117,49 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>26.66817974087171</v>
+        <v>40.00908294799905</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>22.66585678799906</v>
+        <v>19.24325210478369</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.9613527360345413</v>
+        <v>0.3984613648528562</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M107" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-12.71219064454689</v>
+        <v>-1.395478721426864</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>5328</v>
+        <v>5289</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>華容</t>
+          <t>宜鼎</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>367.3569103892326</v>
+        <v>369.5531730137179</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>50.1</v>
+        <v>1065</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,49 +6170,49 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>34.5577817560788</v>
+        <v>26.66817974087171</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>16.24835051664682</v>
+        <v>22.66585678799906</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.4548212397948666</v>
+        <v>0.9613527360345413</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L108" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M108" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.4405644328275014</v>
+        <v>-12.71219064454689</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6127</v>
+        <v>5328</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>九豪</t>
+          <t>華容</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>365.9884171044798</v>
+        <v>367.3569103892326</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>56</v>
+        <v>50.1</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>48.60195894071038</v>
+        <v>34.5577817560788</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>30.33074268352621</v>
+        <v>16.24835051664682</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.4063664207358298</v>
+        <v>0.4548212397948666</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.4313836658553956</v>
+        <v>-0.4405644328275014</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6113</v>
+        <v>6127</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>亞矽</t>
+          <t>九豪</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>365.8298828224281</v>
+        <v>365.9884171044798</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>22.75</v>
+        <v>56</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>45.82001233220766</v>
+        <v>48.60195894071038</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>23.88250123837748</v>
+        <v>30.33074268352621</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.7588529169742557</v>
+        <v>0.4063664207358298</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.08853583828602246</v>
+        <v>-0.4313836658553956</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>4973</v>
+        <v>6113</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>廣穎</t>
+          <t>亞矽</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>364.9939452106959</v>
+        <v>365.8298828224281</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>132.5</v>
+        <v>22.75</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>39.89940563797986</v>
+        <v>45.82001233220766</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.83643441739304</v>
+        <v>23.88250123837748</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.6176754398396934</v>
+        <v>0.7588529169742557</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.6923510208053419</v>
+        <v>-0.08853583828602246</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>4977</v>
+        <v>4973</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>眾達-KY</t>
+          <t>廣穎</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>364.2427140738565</v>
+        <v>364.9939452106959</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>165</v>
+        <v>132.5</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.68092201619593</v>
+        <v>39.89940563797986</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>25.40918254008711</v>
+        <v>16.83643441739304</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.8533687089202689</v>
+        <v>0.6176754398396934</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-1.355937886969279</v>
+        <v>-0.6923510208053419</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>4919</v>
+        <v>4977</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>新唐</t>
+          <t>眾達-KY</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>363.9683145048958</v>
+        <v>364.2427140738565</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>134.5</v>
+        <v>165</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.30845751529743</v>
+        <v>44.68092201619593</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>27.00294425094492</v>
+        <v>25.40918254008711</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.4161983283834993</v>
+        <v>0.8533687089202689</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-2.225607501952393</v>
+        <v>-1.355937886969279</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6463,21 +6463,21 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>4440</v>
+        <v>4919</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>宜新實業</t>
+          <t>新唐</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>362.9973659840693</v>
+        <v>363.9683145048958</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>17.25</v>
+        <v>134.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>39.88737825196014</v>
+        <v>47.30845751529743</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>24.11006520746886</v>
+        <v>27.00294425094492</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>8.272854895619856</v>
+        <v>0.4161983283834993</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.01701825933808096</v>
+        <v>-2.225607501952393</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>volume_break, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6143</v>
+        <v>4440</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>振曜</t>
+          <t>宜新實業</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>362.9814568597225</v>
+        <v>362.9973659840693</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>77.5</v>
+        <v>17.25</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>36.10770157219012</v>
+        <v>39.88737825196014</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>29.78344146172363</v>
+        <v>24.11006520746886</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.5116180035179756</v>
+        <v>8.272854895619856</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.2155590457171543</v>
+        <v>-0.01701825933808096</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
+          <t>volume_break, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6104</v>
+        <v>6143</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>創惟</t>
+          <t>振曜</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>361.7225533573798</v>
+        <v>362.9814568597225</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>85.5</v>
+        <v>77.5</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>36.73633152070484</v>
+        <v>36.10770157219012</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>29.72570408328576</v>
+        <v>29.78344146172363</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.8360942421390062</v>
+        <v>0.5116180035179756</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1273804243687129</v>
+        <v>0.2155590457171543</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6622,21 +6622,21 @@
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>5353</v>
+        <v>6104</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>台林</t>
+          <t>創惟</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>360.7744839129663</v>
+        <v>361.7225533573798</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>27.7</v>
+        <v>85.5</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>41.80378245112596</v>
+        <v>36.73633152070484</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>24.25112705785707</v>
+        <v>29.72570408328576</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4769226661557043</v>
+        <v>0.8360942421390062</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.1174176892242131</v>
+        <v>-0.1273804243687129</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, adx_trending, stronger_than_market</t>
+          <t>avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>4807</v>
+        <v>5353</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>日成-KY</t>
+          <t>台林</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>360.4745727874168</v>
+        <v>360.7744839129663</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>29.85</v>
+        <v>27.7</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>43.29614113421708</v>
+        <v>41.80378245112596</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>36.35255517996109</v>
+        <v>24.25112705785707</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.6722622073423188</v>
+        <v>0.4769226661557043</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1503559539421113</v>
+        <v>-0.1174176892242131</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, adx_trending, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>4438</v>
+        <v>4807</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>廣越</t>
+          <t>日成-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>359.8654926641364</v>
+        <v>360.4745727874168</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>57.4</v>
+        <v>29.85</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>50.35706778291946</v>
+        <v>43.29614113421708</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>13.5770171040361</v>
+        <v>36.35255517996109</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.6802728493950591</v>
+        <v>0.6722622073423188</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.1948126185404503</v>
+        <v>-0.1503559539421113</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>5274</v>
+        <v>4438</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>信驊</t>
+          <t>廣越</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>358.1433075754226</v>
+        <v>359.8654926641364</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>16010</v>
+        <v>57.4</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>39.50698523648437</v>
+        <v>50.35706778291946</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>18.69857287022019</v>
+        <v>13.5770171040361</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.8402950493068254</v>
+        <v>0.6802728493950591</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-308.7511184161173</v>
+        <v>0.1948126185404503</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market</t>
+          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>4306</v>
+        <v>5274</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>炎洲</t>
+          <t>信驊</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>357.0404885708268</v>
+        <v>358.1433075754226</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>14.55</v>
+        <v>16010</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>46.78930828391849</v>
+        <v>39.50698523648437</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>12.15487796564395</v>
+        <v>18.69857287022019</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.195579007307682</v>
+        <v>0.8402950493068254</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.03203118802256804</v>
+        <v>-308.7511184161173</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, stronger_than_market, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>5452</v>
+        <v>4306</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>佶優</t>
+          <t>炎洲</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>356.0323217098795</v>
+        <v>357.0404885708268</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>27.7</v>
+        <v>14.55</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>46.30494908083674</v>
+        <v>46.78930828391849</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>15.48152845522575</v>
+        <v>12.15487796564395</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.3015382345052691</v>
+        <v>1.195579007307682</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.2304632462328572</v>
+        <v>0.03203118802256804</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, avoid_chase, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>4576</v>
+        <v>5452</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>大銀微系統</t>
+          <t>佶優</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>350.0709830223309</v>
+        <v>356.0323217098795</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>203.5</v>
+        <v>27.7</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>38.86091233231943</v>
+        <v>46.30494908083674</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>17.47626217898176</v>
+        <v>15.48152845522575</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.6142024426889214</v>
+        <v>0.3015382345052691</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-3.057272921674938</v>
+        <v>-0.2304632462328572</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market</t>
+          <t>avoid_chase, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>5481</v>
+        <v>4576</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>新華</t>
+          <t>大銀微系統</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>346.6115643256794</v>
+        <v>350.0709830223309</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>20.8</v>
+        <v>203.5</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>46.92634526818705</v>
+        <v>38.86091233231943</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>21.16676000470757</v>
+        <v>17.47626217898176</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.7138156803899786</v>
+        <v>0.6142024426889214</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.05089014203254998</v>
+        <v>-3.057272921674938</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, avoid_chase, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>4542</v>
+        <v>5481</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>科嶠</t>
+          <t>新華</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>344.9208084580185</v>
+        <v>346.6115643256794</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>345</v>
+        <v>20.8</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,16 +7071,16 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>52.02037517836654</v>
+        <v>46.92634526818705</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>31.1840202936802</v>
+        <v>21.16676000470757</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>1.180801934696807</v>
+        <v>0.7138156803899786</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L125" s="2" t="n">
         <v>0</v>
@@ -7089,11 +7089,11 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.5544916635051713</v>
+        <v>-0.05089014203254998</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>avoid_chase, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -7654,13 +7654,13 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>50.98254542919024</v>
+        <v>50.98254623120573</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>12.88298221159421</v>
+        <v>12.88298105143169</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.4696971423362654</v>
+        <v>0.4696971423362655</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>1</v>
@@ -7672,11 +7672,11 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-0.757762094905793</v>
+        <v>-0.7577621028251968</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
scan: seg4 2026-10-26 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq5_2026-10-22.xlsx
@@ -658,7 +658,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>76.68149937272629</v>
+        <v>76.68149939128861</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>45.14922240515013</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.633135905664997</v>
+        <v>0.63313590558712</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>75.62781152768241</v>
+        <v>75.62781158286103</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>33.23024401640993</v>
+        <v>33.23024410910637</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>8.88771491122071</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.6296485314236735</v>
+        <v>0.6296485310083586</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>60.62619341691623</v>
+        <v>60.62619349720432</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14.32924373843882</v>
+        <v>14.32924373459093</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>2.194768667348381</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.0865152320444014</v>
+        <v>0.0865152319795085</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59.47928272059173</v>
+        <v>59.47928266939027</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>45.41498955465588</v>
+        <v>45.41498957728069</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.63114564809902</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.8856934923379711</v>
+        <v>0.8856934951932836</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>76.97465595948282</v>
+        <v>76.9746559621442</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>46.87453176747054</v>
+        <v>46.87453181059919</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.366496525594463</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2904629831533589</v>
+        <v>0.2904629831793186</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>65.67868300890024</v>
+        <v>65.67868302410197</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>30.53779738829009</v>
+        <v>30.53779742739253</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>0.8349163115252451</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.1341545466372664</v>
+        <v>0.1341545466632272</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>820.3084367009719</v>
+        <v>820.3084367009718</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>211</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>71.5700034326542</v>
+        <v>71.57000353111158</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>36.78282114826709</v>
+        <v>36.78282122420052</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>0.8913805972871407</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.570795598641013</v>
+        <v>2.570795597862289</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>819.3531347689857</v>
+        <v>819.3531347689856</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>357.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55.96038896170143</v>
+        <v>55.96038883967484</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>23.48573574731696</v>
+        <v>23.48573592595485</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.8701307681813</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.1003863061829637</v>
+        <v>0.1003863107254839</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>679.3975177197792</v>
+        <v>679.3975177197799</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>11.25</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>60.21347577898206</v>
+        <v>60.21347570832118</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>31.00240523372722</v>
+        <v>31.00240526322215</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.042096312472886</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.008983992564672277</v>
+        <v>0.008983992538712959</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>660.5095987043072</v>
+        <v>660.509598704304</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>55.5</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>72.07577644182594</v>
+        <v>72.07577657735781</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>33.77864127782711</v>
+        <v>33.77864129434838</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.9923866713990172</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.5747915023866055</v>
+        <v>0.5747915022049064</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>50.27586256473572</v>
+        <v>50.27586248194106</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>22.56074183252831</v>
+        <v>22.56074181610573</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.7390053598164795</v>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>536.9736145630038</v>
+        <v>536.9736145630039</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>364</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>40.18949052352819</v>
+        <v>40.18949045887918</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>17.3784076792905</v>
+        <v>17.3784076482947</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.9249136326467248</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.2580446870492938</v>
+        <v>0.2580446862705221</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>518.9270415728869</v>
+        <v>518.9270415728873</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>99.40000000000001</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>56.61904501304829</v>
+        <v>56.6190449488293</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>15.14496074386768</v>
+        <v>15.14496083176113</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.1855148505574815</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.3696761323097785</v>
+        <v>0.3696761326731772</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>44.30577872897049</v>
+        <v>44.30577881213096</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>22.39514195157125</v>
+        <v>22.39514198317853</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.6447890569664552</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.3072155041532131</v>
+        <v>-0.3072155046204466</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>512.3323149655887</v>
+        <v>512.3323149655886</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>59.9</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>64.79588090891821</v>
+        <v>64.79588087499363</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>18.20922777055821</v>
+        <v>18.2092277303493</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>1.431497212872433</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.3572211632381573</v>
+        <v>0.3572211634717797</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>511.2690813201278</v>
+        <v>511.2690813201277</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>8.15</v>
@@ -3629,7 +3629,7 @@
         <v>58.0782696013524</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>33.71893242993304</v>
+        <v>33.7189325155826</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.3850333605444601</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.04968643677562544</v>
+        <v>0.04968643678860343</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>47.79901958576991</v>
+        <v>47.7990196217601</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>26.90108525454476</v>
+        <v>26.90108527806225</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.5099353439296239</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.07018423169658501</v>
+        <v>-0.07018423172253849</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>50.83164753232131</v>
+        <v>50.83164770611015</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>13.07000880313028</v>
+        <v>13.07000878649525</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.4831670608026585</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.004001053808981858</v>
+        <v>0.004001053679199146</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>51.11663425678567</v>
+        <v>51.11663392127251</v>
       </c>
       <c r="I71" s="2" t="n">
         <v>28.06804479609417</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-0.01594288378441305</v>
+        <v>-0.01594288371952016</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>52.5769108060732</v>
+        <v>52.57691108752931</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>32.92473625424009</v>
+        <v>32.92473637139329</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.7582957866777388</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.07527013378316916</v>
+        <v>-0.07527013412062233</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>51.51804692554725</v>
+        <v>51.51804698664864</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>8.429310534968556</v>
+        <v>8.429310652571086</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>3.787550729720638</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.8031848987410348</v>
+        <v>0.8031848981959255</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>51.15867346009517</v>
+        <v>51.15867334035647</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>17.30889587597311</v>
+        <v>17.30889586887792</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5547209661035036</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.0622894751379249</v>
+        <v>-0.06228947508600841</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>55.46918353695793</v>
+        <v>55.46918347114671</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>14.24548215306085</v>
+        <v>14.24548221231429</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.6460041308695501</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.7925144962944661</v>
+        <v>0.7925144947370286</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>52.70391104792866</v>
+        <v>52.70391121384832</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>12.30888442507745</v>
+        <v>12.3088843864571</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.9233647726624306</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>0.2038132078206641</v>
+        <v>0.2038132077687497</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>46.62616352667133</v>
+        <v>46.62616352827739</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>20.74162651487287</v>
+        <v>20.74162666623761</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.4878336344862177</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-3.566679099418293</v>
+        <v>-3.566679099496168</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>49.27639964223666</v>
+        <v>49.27639970309146</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>14.03993738986184</v>
+        <v>14.03993747607021</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.5821020311408892</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1706137507478546</v>
+        <v>-0.1706137523053128</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>408.8057594870941</v>
+        <v>408.805759487094</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>120</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>47.96259856797898</v>
+        <v>47.96259845952477</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>30.19699358240646</v>
+        <v>30.19699377374975</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.7298314301957985</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.4364919034771391</v>
+        <v>-0.4364919030877787</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>53.38968367484803</v>
+        <v>53.38968375421145</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>34.24851127541276</v>
+        <v>34.24851117496686</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.4439585338242862</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.04489292534735034</v>
+        <v>-0.04489292555500801</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>382.9793271361722</v>
+        <v>382.9793271361729</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>13.9</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>48.02327140648779</v>
+        <v>48.02327146745171</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.54492496431556</v>
+        <v>16.54492504018516</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>1.41489103612369</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.006273682245060475</v>
+        <v>-0.006273682258038859</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>365.9884171044798</v>
+        <v>365.98841710448</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>56</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>48.60195894071038</v>
+        <v>48.60195893895624</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>30.33074268352621</v>
+        <v>30.33074285594414</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.4063664207358298</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.4313836658553956</v>
+        <v>-0.4313836660500758</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.88737825196014</v>
+        <v>39.88737906873644</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>24.11006520746886</v>
+        <v>24.11006533264294</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>8.272854895619856</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.01701825933808096</v>
+        <v>-0.01701825940297361</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>362.9814568597225</v>
+        <v>362.9814568597226</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>77.5</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>36.10770157219012</v>
+        <v>36.10770209157645</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>29.78344146172363</v>
+        <v>29.78344173421315</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.5116180035179756</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.2155590457171543</v>
+        <v>0.2155590455873644</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6809,7 +6809,7 @@
         <v>43.29614113421708</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>36.35255517996109</v>
+        <v>36.35255525013297</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.6722622073423188</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.1503559539421113</v>
+        <v>-0.1503559539680676</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>50.35706778291946</v>
+        <v>50.35706788253953</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>13.5770171040361</v>
+        <v>13.57701706049791</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.6802728493950591</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.1948126185404503</v>
+        <v>0.1948126186961989</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>357.0404885708268</v>
+        <v>357.0404885708269</v>
       </c>
       <c r="E123" s="2" t="n">
         <v>14.55</v>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>46.78930828391849</v>
+        <v>46.78930895770316</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>12.15487796564395</v>
+        <v>12.15487846760463</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>1.195579007307682</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.03203118802256804</v>
+        <v>0.03203118767214329</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>350.0709830223309</v>
+        <v>350.0709830223308</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>203.5</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>38.86091233231943</v>
+        <v>38.86091233645045</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>17.47626217898176</v>
+        <v>17.47626224086993</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6142024426889214</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-3.057272921674938</v>
+        <v>-3.057272922323866</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>341.8387145284736</v>
+        <v>341.8387145284734</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>29.55</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>42.96597753953057</v>
+        <v>42.96597771954704</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>14.62376239352439</v>
+        <v>14.62376240648946</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.7130579007116358</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.02347671882425922</v>
+        <v>-0.02347671926553602</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>32.68427999236286</v>
+        <v>32.68427999059814</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>23.52919278182889</v>
+        <v>23.52919271087001</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.6805581984820145</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-2.106051157790574</v>
+        <v>-2.106051157816541</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7428,7 +7428,7 @@
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>331.2684445312723</v>
+        <v>331.2684445312724</v>
       </c>
       <c r="E132" s="2" t="n">
         <v>17.35</v>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>43.97152451736815</v>
+        <v>43.97152442225895</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>26.5019938760811</v>
+        <v>26.50199400367705</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>1.299959538459392</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>-0.05060202006788389</v>
+        <v>-0.05060202005490327</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7481,7 +7481,7 @@
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>330.0188053483457</v>
+        <v>330.0188053483462</v>
       </c>
       <c r="E133" s="2" t="n">
         <v>243</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>31.59402175225597</v>
+        <v>31.59402178107958</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>22.63182042070134</v>
+        <v>22.63182047103385</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>0.6827601605186143</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-2.267224429641066</v>
+        <v>-2.267224430549573</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>37.8789187578731</v>
+        <v>37.87891870645439</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>21.59516848943016</v>
+        <v>21.59516850105849</v>
       </c>
       <c r="J135" s="2" t="n">
         <v>1.407121613476874</v>
@@ -7619,7 +7619,7 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>0.06484927815292385</v>
+        <v>0.06484927817888309</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
@@ -7707,10 +7707,10 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>43.29297622419337</v>
+        <v>43.29297635664287</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>8.219450223861772</v>
+        <v>8.219450362409731</v>
       </c>
       <c r="J137" s="2" t="n">
         <v>1.608802507767971</v>
@@ -7725,7 +7725,7 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-0.0871775332778178</v>
+        <v>-0.08717753345951917</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>317.1810020708892</v>
+        <v>317.1810020708893</v>
       </c>
       <c r="E140" s="2" t="n">
         <v>151</v>
@@ -7869,7 +7869,7 @@
         <v>38.90157884293632</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>13.09245221813323</v>
+        <v>13.09245228899301</v>
       </c>
       <c r="J140" s="2" t="n">
         <v>1.229683437388532</v>
@@ -7884,7 +7884,7 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>-0.2070163762059507</v>
+        <v>-0.2070163768548829</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
@@ -8184,10 +8184,10 @@
         <v>0</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>31.63628999067996</v>
+        <v>31.63629005924344</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>34.31628238265345</v>
+        <v>34.31628268745065</v>
       </c>
       <c r="J146" s="2" t="n">
         <v>0.887391424643281</v>
@@ -8202,7 +8202,7 @@
         <v>-1</v>
       </c>
       <c r="N146" s="2" t="n">
-        <v>-0.1456006134905978</v>
+        <v>-0.145600613581446</v>
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>41.6995325267193</v>
+        <v>41.69953257746329</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>20.65128753393996</v>
+        <v>20.6512873971563</v>
       </c>
       <c r="J147" s="2" t="n">
         <v>1.382959415199727</v>
@@ -8255,7 +8255,7 @@
         <v>-1</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>-0.1441741153319445</v>
+        <v>-0.1441741155915168</v>
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
@@ -8276,7 +8276,7 @@
         <v/>
       </c>
       <c r="D148" s="2" t="n">
-        <v>303.1645245542138</v>
+        <v>303.1645245542201</v>
       </c>
       <c r="E148" s="2" t="n">
         <v>41.4</v>
@@ -8290,10 +8290,10 @@
         <v>0</v>
       </c>
       <c r="H148" s="2" t="n">
-        <v>42.78363958655368</v>
+        <v>42.78363911682035</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>10.29812823698929</v>
+        <v>10.29812863384183</v>
       </c>
       <c r="J148" s="2" t="n">
         <v>0.802734428693174</v>
@@ -8308,7 +8308,7 @@
         <v>-1</v>
       </c>
       <c r="N148" s="2" t="n">
-        <v>0.1049144656030342</v>
+        <v>0.1049144660183574</v>
       </c>
       <c r="O148" s="2" t="inlineStr">
         <is>
@@ -8435,7 +8435,7 @@
         <v/>
       </c>
       <c r="D151" s="2" t="n">
-        <v>301.101442559547</v>
+        <v>301.1014425595482</v>
       </c>
       <c r="E151" s="2" t="n">
         <v>43.1</v>
@@ -8449,10 +8449,10 @@
         <v>0</v>
       </c>
       <c r="H151" s="2" t="n">
-        <v>31.06503230071679</v>
+        <v>31.06503221509364</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>22.37541242533272</v>
+        <v>22.37541240790502</v>
       </c>
       <c r="J151" s="2" t="n">
         <v>1.083936085743771</v>
@@ -8467,7 +8467,7 @@
         <v>-1</v>
       </c>
       <c r="N151" s="2" t="n">
-        <v>-0.08439440632358189</v>
+        <v>-0.08439440642741591</v>
       </c>
       <c r="O151" s="2" t="inlineStr">
         <is>
@@ -8488,7 +8488,7 @@
         <v/>
       </c>
       <c r="D152" s="2" t="n">
-        <v>299.7877468443463</v>
+        <v>299.7877468443464</v>
       </c>
       <c r="E152" s="2" t="n">
         <v>45.9</v>
@@ -8502,10 +8502,10 @@
         <v>0</v>
       </c>
       <c r="H152" s="2" t="n">
-        <v>44.90336016766504</v>
+        <v>44.9033601801099</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>14.60590485366819</v>
+        <v>14.60590489219861</v>
       </c>
       <c r="J152" s="2" t="n">
         <v>0.4365467663627698</v>
@@ -8520,7 +8520,7 @@
         <v>-1</v>
       </c>
       <c r="N152" s="2" t="n">
-        <v>-0.03115178347043324</v>
+        <v>-0.03115178398957852</v>
       </c>
       <c r="O152" s="2" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         <v/>
       </c>
       <c r="D153" s="2" t="n">
-        <v>299.3078248505359</v>
+        <v>299.3078248505356</v>
       </c>
       <c r="E153" s="2" t="n">
         <v>33.65</v>
@@ -8555,10 +8555,10 @@
         <v>0</v>
       </c>
       <c r="H153" s="2" t="n">
-        <v>36.42773796874001</v>
+        <v>36.42773810103204</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>16.68757537318828</v>
+        <v>16.68757543423608</v>
       </c>
       <c r="J153" s="2" t="n">
         <v>1.002064306895856</v>
@@ -8573,7 +8573,7 @@
         <v>-1</v>
       </c>
       <c r="N153" s="2" t="n">
-        <v>-0.1176635399168415</v>
+        <v>-0.1176635401893956</v>
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
@@ -8594,7 +8594,7 @@
         <v/>
       </c>
       <c r="D154" s="2" t="n">
-        <v>297.2168235865824</v>
+        <v>297.2168235865809</v>
       </c>
       <c r="E154" s="2" t="n">
         <v>30.6</v>
@@ -8608,10 +8608,10 @@
         <v>0</v>
       </c>
       <c r="H154" s="2" t="n">
-        <v>40.31674026370486</v>
+        <v>40.31674032282429</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>13.66220137761545</v>
+        <v>13.66220146518656</v>
       </c>
       <c r="J154" s="2" t="n">
         <v>0.6114705285630955</v>
@@ -8626,7 +8626,7 @@
         <v>-1</v>
       </c>
       <c r="N154" s="2" t="n">
-        <v>-0.2071251976386767</v>
+        <v>-0.2071251976905887</v>
       </c>
       <c r="O154" s="2" t="inlineStr">
         <is>
@@ -8806,7 +8806,7 @@
         <v/>
       </c>
       <c r="D158" s="2" t="n">
-        <v>293.1621971619021</v>
+        <v>293.1621971619023</v>
       </c>
       <c r="E158" s="2" t="n">
         <v>153.5</v>
@@ -8820,10 +8820,10 @@
         <v>0</v>
       </c>
       <c r="H158" s="2" t="n">
-        <v>28.20510512261724</v>
+        <v>28.20510521227703</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>32.74862504386115</v>
+        <v>32.74862519851375</v>
       </c>
       <c r="J158" s="2" t="n">
         <v>0.6936514497967526</v>
@@ -8838,7 +8838,7 @@
         <v>-1</v>
       </c>
       <c r="N158" s="2" t="n">
-        <v>-0.3838384793408052</v>
+        <v>-0.3838384799897012</v>
       </c>
       <c r="O158" s="2" t="inlineStr">
         <is>
@@ -8965,7 +8965,7 @@
         <v/>
       </c>
       <c r="D161" s="2" t="n">
-        <v>291.7270963132805</v>
+        <v>291.7270963132811</v>
       </c>
       <c r="E161" s="2" t="n">
         <v>4.38</v>
@@ -8979,10 +8979,10 @@
         <v>0</v>
       </c>
       <c r="H161" s="2" t="n">
-        <v>22.04402382834164</v>
+        <v>22.04402369860804</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>33.59318349614129</v>
+        <v>33.59318342434285</v>
       </c>
       <c r="J161" s="2" t="n">
         <v>1.008638454187074</v>
@@ -8997,7 +8997,7 @@
         <v>-1</v>
       </c>
       <c r="N161" s="2" t="n">
-        <v>-0.02607761003398468</v>
+        <v>-0.02607761001581436</v>
       </c>
       <c r="O161" s="2" t="inlineStr">
         <is>
@@ -9085,10 +9085,10 @@
         <v>0</v>
       </c>
       <c r="H163" s="2" t="n">
-        <v>36.64427089391443</v>
+        <v>36.64427094645512</v>
       </c>
       <c r="I163" s="2" t="n">
-        <v>14.16181574010007</v>
+        <v>14.16181572660594</v>
       </c>
       <c r="J163" s="2" t="n">
         <v>1.406986597668995</v>
@@ -9103,7 +9103,7 @@
         <v>-1</v>
       </c>
       <c r="N163" s="2" t="n">
-        <v>-0.001308485747722007</v>
+        <v>-0.001308485760699848</v>
       </c>
       <c r="O163" s="2" t="inlineStr">
         <is>
@@ -9124,7 +9124,7 @@
         <v/>
       </c>
       <c r="D164" s="2" t="n">
-        <v>286.5271075486057</v>
+        <v>286.5271075486029</v>
       </c>
       <c r="E164" s="2" t="n">
         <v>24.85</v>
@@ -9138,10 +9138,10 @@
         <v>0</v>
       </c>
       <c r="H164" s="2" t="n">
-        <v>22.80208346969862</v>
+        <v>22.80208347791597</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>24.6078278044827</v>
+        <v>24.60782782540012</v>
       </c>
       <c r="J164" s="2" t="n">
         <v>1.153957023328669</v>
@@ -9156,7 +9156,7 @@
         <v>-1</v>
       </c>
       <c r="N164" s="2" t="n">
-        <v>-0.3270672715967458</v>
+        <v>-0.3270672717005738</v>
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
@@ -9191,10 +9191,10 @@
         <v>0</v>
       </c>
       <c r="H165" s="2" t="n">
-        <v>29.70378164673039</v>
+        <v>29.70378172007359</v>
       </c>
       <c r="I165" s="2" t="n">
-        <v>19.39937031628117</v>
+        <v>19.39937038033904</v>
       </c>
       <c r="J165" s="2" t="n">
         <v>1.11402853334793</v>
@@ -9209,7 +9209,7 @@
         <v>-1</v>
       </c>
       <c r="N165" s="2" t="n">
-        <v>-0.0666189123922587</v>
+        <v>-0.06661891252203955</v>
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
@@ -9300,7 +9300,7 @@
         <v>42.82428873352998</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>21.6357354266385</v>
+        <v>21.63573551810554</v>
       </c>
       <c r="J167" s="2" t="n">
         <v>0.4778419857539952</v>
@@ -9315,7 +9315,7 @@
         <v>-1</v>
       </c>
       <c r="N167" s="2" t="n">
-        <v>-0.1023583394919087</v>
+        <v>-0.1023583395568006</v>
       </c>
       <c r="O167" s="2" t="inlineStr">
         <is>
@@ -9389,7 +9389,7 @@
         <v/>
       </c>
       <c r="D169" s="2" t="n">
-        <v>276.6961310129745</v>
+        <v>276.6961310129743</v>
       </c>
       <c r="E169" s="2" t="n">
         <v>156.5</v>
@@ -9403,10 +9403,10 @@
         <v>0</v>
       </c>
       <c r="H169" s="2" t="n">
-        <v>41.25478929353587</v>
+        <v>41.25478935832528</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>17.11739797128961</v>
+        <v>17.11739789259614</v>
       </c>
       <c r="J169" s="2" t="n">
         <v>0.2436837385676321</v>
@@ -9421,7 +9421,7 @@
         <v>-1</v>
       </c>
       <c r="N169" s="2" t="n">
-        <v>-2.382570721149186</v>
+        <v>-2.382570723615143</v>
       </c>
       <c r="O169" s="2" t="inlineStr">
         <is>
@@ -9495,7 +9495,7 @@
         <v/>
       </c>
       <c r="D171" s="2" t="n">
-        <v>272.0832488391526</v>
+        <v>272.0832488391529</v>
       </c>
       <c r="E171" s="2" t="n">
         <v>14.85</v>
@@ -9509,10 +9509,10 @@
         <v>0</v>
       </c>
       <c r="H171" s="2" t="n">
-        <v>46.54980906255457</v>
+        <v>46.54980902841746</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>30.54367779188036</v>
+        <v>30.54367776891876</v>
       </c>
       <c r="J171" s="2" t="n">
         <v>0.3666652127361422</v>
@@ -9527,7 +9527,7 @@
         <v>-1</v>
       </c>
       <c r="N171" s="2" t="n">
-        <v>-0.1396944742212619</v>
+        <v>-0.1396944742082832</v>
       </c>
       <c r="O171" s="2" t="inlineStr">
         <is>
@@ -9548,7 +9548,7 @@
         <v/>
       </c>
       <c r="D172" s="2" t="n">
-        <v>271.3702774210973</v>
+        <v>271.3702774210974</v>
       </c>
       <c r="E172" s="2" t="n">
         <v>15.55</v>
@@ -9562,10 +9562,10 @@
         <v>0</v>
       </c>
       <c r="H172" s="2" t="n">
-        <v>40.98131002297067</v>
+        <v>40.98130881542331</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>13.52910290587363</v>
+        <v>13.52910293441596</v>
       </c>
       <c r="J172" s="2" t="n">
         <v>0.5369198402571415</v>
@@ -9580,7 +9580,7 @@
         <v>-1</v>
       </c>
       <c r="N172" s="2" t="n">
-        <v>-0.01772146793516577</v>
+        <v>-0.0177214674549534</v>
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
@@ -9774,10 +9774,10 @@
         <v>0</v>
       </c>
       <c r="H176" s="2" t="n">
-        <v>28.20356584881408</v>
+        <v>28.20356627988222</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>25.03071016243477</v>
+        <v>25.03071016284836</v>
       </c>
       <c r="J176" s="2" t="n">
         <v>1.62639351202384</v>
@@ -9792,7 +9792,7 @@
         <v>-1</v>
       </c>
       <c r="N176" s="2" t="n">
-        <v>-0.7996520314730744</v>
+        <v>-0.7996520317326525</v>
       </c>
       <c r="O176" s="2" t="inlineStr">
         <is>
@@ -9919,7 +9919,7 @@
         <v/>
       </c>
       <c r="D179" s="2" t="n">
-        <v>260.8700133617154</v>
+        <v>260.8700133617155</v>
       </c>
       <c r="E179" s="2" t="n">
         <v>79.2</v>
@@ -9933,10 +9933,10 @@
         <v>0</v>
       </c>
       <c r="H179" s="2" t="n">
-        <v>26.20987218977669</v>
+        <v>26.20987221564319</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>24.89834203370151</v>
+        <v>24.8983420444726</v>
       </c>
       <c r="J179" s="2" t="n">
         <v>1.084903534857465</v>
@@ -9951,7 +9951,7 @@
         <v>-1</v>
       </c>
       <c r="N179" s="2" t="n">
-        <v>-0.9670179704384623</v>
+        <v>-0.9670179707758968</v>
       </c>
       <c r="O179" s="2" t="inlineStr">
         <is>
@@ -10039,10 +10039,10 @@
         <v>0</v>
       </c>
       <c r="H181" s="2" t="n">
-        <v>38.54461901707173</v>
+        <v>38.54461907017079</v>
       </c>
       <c r="I181" s="2" t="n">
-        <v>40.75108805797031</v>
+        <v>40.75108797824153</v>
       </c>
       <c r="J181" s="2" t="n">
         <v>0.9614105986484248</v>
@@ -10057,7 +10057,7 @@
         <v>-1</v>
       </c>
       <c r="N181" s="2" t="n">
-        <v>0.03981647062061794</v>
+        <v>0.03981647054274395</v>
       </c>
       <c r="O181" s="2" t="inlineStr">
         <is>
@@ -10502,7 +10502,7 @@
         <v/>
       </c>
       <c r="D190" s="2" t="n">
-        <v>220.3156365324373</v>
+        <v>220.3156365324376</v>
       </c>
       <c r="E190" s="2" t="n">
         <v>24.05</v>
@@ -10516,10 +10516,10 @@
         <v>0</v>
       </c>
       <c r="H190" s="2" t="n">
-        <v>44.1394836091353</v>
+        <v>44.13948359426268</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>17.05315844375646</v>
+        <v>17.05315849245809</v>
       </c>
       <c r="J190" s="2" t="n">
         <v>0.7398912444334981</v>
@@ -10534,7 +10534,7 @@
         <v>-1</v>
       </c>
       <c r="N190" s="2" t="n">
-        <v>-0.06590060817949145</v>
+        <v>-0.065900608244384</v>
       </c>
       <c r="O190" s="2" t="inlineStr">
         <is>
@@ -10622,10 +10622,10 @@
         <v>0</v>
       </c>
       <c r="H192" s="2" t="n">
-        <v>36.58491632774265</v>
+        <v>36.58491631652067</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>9.037833094262629</v>
+        <v>9.037833106550245</v>
       </c>
       <c r="J192" s="2" t="n">
         <v>0.6697783347547684</v>
@@ -10640,7 +10640,7 @@
         <v>-1</v>
       </c>
       <c r="N192" s="2" t="n">
-        <v>-0.03385995130727137</v>
+        <v>-0.03385995141110609</v>
       </c>
       <c r="O192" s="2" t="inlineStr">
         <is>
@@ -10728,10 +10728,10 @@
         <v>0</v>
       </c>
       <c r="H194" s="2" t="n">
-        <v>41.83001349954603</v>
+        <v>41.830013619871</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>15.45808287529983</v>
+        <v>15.45808287236789</v>
       </c>
       <c r="J194" s="2" t="n">
         <v>0.8421638776482366</v>
@@ -10746,7 +10746,7 @@
         <v>-1</v>
       </c>
       <c r="N194" s="2" t="n">
-        <v>0.2463778889072239</v>
+        <v>0.2463778885178594</v>
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
@@ -10781,10 +10781,10 @@
         <v>0</v>
       </c>
       <c r="H195" s="2" t="n">
-        <v>48.18664909491016</v>
+        <v>48.1866490676645</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>3.905845542842978</v>
+        <v>3.905845599310196</v>
       </c>
       <c r="J195" s="2" t="n">
         <v>0.9426545961799387</v>
@@ -10820,7 +10820,7 @@
         <v/>
       </c>
       <c r="D196" s="2" t="n">
-        <v>213.4095685434217</v>
+        <v>213.4095685434212</v>
       </c>
       <c r="E196" s="2" t="n">
         <v>42.3</v>
@@ -10834,10 +10834,10 @@
         <v>0</v>
       </c>
       <c r="H196" s="2" t="n">
-        <v>37.92450671951065</v>
+        <v>37.92450674919996</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>11.06908946609854</v>
+        <v>11.06908946212346</v>
       </c>
       <c r="J196" s="2" t="n">
         <v>1.224654676933049</v>
@@ -10852,7 +10852,7 @@
         <v>-1</v>
       </c>
       <c r="N196" s="2" t="n">
-        <v>-0.04423553569048475</v>
+        <v>-0.04423553574239592</v>
       </c>
       <c r="O196" s="2" t="inlineStr">
         <is>
@@ -10873,7 +10873,7 @@
         <v/>
       </c>
       <c r="D197" s="2" t="n">
-        <v>212.5863762881911</v>
+        <v>212.5863762881918</v>
       </c>
       <c r="E197" s="2" t="n">
         <v>37.95</v>
@@ -10887,10 +10887,10 @@
         <v>0</v>
       </c>
       <c r="H197" s="2" t="n">
-        <v>53.35410051211685</v>
+        <v>53.35410077941022</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>7.705147922586209</v>
+        <v>7.705148449733987</v>
       </c>
       <c r="J197" s="2" t="n">
         <v>1.427156852417571</v>
@@ -10905,7 +10905,7 @@
         <v>-1</v>
       </c>
       <c r="N197" s="2" t="n">
-        <v>2.097575356510142</v>
+        <v>2.097575343557408</v>
       </c>
       <c r="O197" s="2" t="inlineStr">
         <is>
@@ -10979,7 +10979,7 @@
         <v/>
       </c>
       <c r="D199" s="2" t="n">
-        <v>206.8301364027217</v>
+        <v>206.8301364027216</v>
       </c>
       <c r="E199" s="2" t="n">
         <v>13.6</v>
@@ -10993,10 +10993,10 @@
         <v>0</v>
       </c>
       <c r="H199" s="2" t="n">
-        <v>43.5360596698211</v>
+        <v>43.53605871195966</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>16.44698845309259</v>
+        <v>16.44698838277809</v>
       </c>
       <c r="J199" s="2" t="n">
         <v>1.094478665681981</v>
@@ -11011,7 +11011,7 @@
         <v>-1</v>
       </c>
       <c r="N199" s="2" t="n">
-        <v>-0.04430658777172553</v>
+        <v>-0.04430658703770259</v>
       </c>
       <c r="O199" s="2" t="inlineStr">
         <is>
@@ -11046,10 +11046,10 @@
         <v>0</v>
       </c>
       <c r="H200" s="2" t="n">
-        <v>38.5348291992474</v>
+        <v>38.5348294050554</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>19.58658080315357</v>
+        <v>19.58658084782631</v>
       </c>
       <c r="J200" s="2" t="n">
         <v>0.4968376829904354</v>
@@ -11064,7 +11064,7 @@
         <v>-1</v>
       </c>
       <c r="N200" s="2" t="n">
-        <v>0.007071281942231722</v>
+        <v>0.007071281916275471</v>
       </c>
       <c r="O200" s="2" t="inlineStr">
         <is>
@@ -11085,7 +11085,7 @@
         <v/>
       </c>
       <c r="D201" s="2" t="n">
-        <v>204.5901174624759</v>
+        <v>204.5901174624741</v>
       </c>
       <c r="E201" s="2" t="n">
         <v>186.5</v>
@@ -11099,10 +11099,10 @@
         <v>0</v>
       </c>
       <c r="H201" s="2" t="n">
-        <v>40.71256244144305</v>
+        <v>40.71256239369096</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>18.33279562482971</v>
+        <v>18.33279565799631</v>
       </c>
       <c r="J201" s="2" t="n">
         <v>0.3844950592001168</v>
@@ -11117,7 +11117,7 @@
         <v>-1</v>
       </c>
       <c r="N201" s="2" t="n">
-        <v>-2.632630622008804</v>
+        <v>-2.632630622138599</v>
       </c>
       <c r="O201" s="2" t="inlineStr">
         <is>
@@ -11244,7 +11244,7 @@
         <v/>
       </c>
       <c r="D204" s="2" t="n">
-        <v>200.1847741796148</v>
+        <v>200.1847741796149</v>
       </c>
       <c r="E204" s="2" t="n">
         <v>386</v>
@@ -11258,10 +11258,10 @@
         <v>0</v>
       </c>
       <c r="H204" s="2" t="n">
-        <v>33.10934305596221</v>
+        <v>33.10934334559788</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>22.13512999966407</v>
+        <v>22.13512975186148</v>
       </c>
       <c r="J204" s="2" t="n">
         <v>0.6825390353399657</v>
@@ -11276,7 +11276,7 @@
         <v>-1</v>
       </c>
       <c r="N204" s="2" t="n">
-        <v>-0.4739738911186713</v>
+        <v>-0.4739739069526312</v>
       </c>
       <c r="O204" s="2" t="inlineStr">
         <is>
@@ -11364,10 +11364,10 @@
         <v>0</v>
       </c>
       <c r="H206" s="2" t="n">
-        <v>41.71395684591754</v>
+        <v>41.71395701265217</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>18.37140671629109</v>
+        <v>18.37140674472566</v>
       </c>
       <c r="J206" s="2" t="n">
         <v>0.8461952155823232</v>
@@ -11382,7 +11382,7 @@
         <v>-1</v>
       </c>
       <c r="N206" s="2" t="n">
-        <v>0.02166942211000322</v>
+        <v>0.021669421902346</v>
       </c>
       <c r="O206" s="2" t="inlineStr">
         <is>
@@ -11417,10 +11417,10 @@
         <v>0</v>
       </c>
       <c r="H207" s="2" t="n">
-        <v>35.57084624585241</v>
+        <v>35.5708463310456</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>22.85075977211238</v>
+        <v>22.85075978968998</v>
       </c>
       <c r="J207" s="2" t="n">
         <v>1.112741633940383</v>
@@ -11435,7 +11435,7 @@
         <v>-1</v>
       </c>
       <c r="N207" s="2" t="n">
-        <v>-0.3015063018474607</v>
+        <v>-0.3015063019642711</v>
       </c>
       <c r="O207" s="2" t="inlineStr">
         <is>
@@ -11629,10 +11629,10 @@
         <v>0</v>
       </c>
       <c r="H211" s="2" t="n">
-        <v>42.0340771902471</v>
+        <v>42.03407714117843</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>12.9906915380676</v>
+        <v>12.99069154877616</v>
       </c>
       <c r="J211" s="2" t="n">
         <v>0.6439795234793296</v>
@@ -11647,7 +11647,7 @@
         <v>-1</v>
       </c>
       <c r="N211" s="2" t="n">
-        <v>-0.1065072559501609</v>
+        <v>-0.1065072558203785</v>
       </c>
       <c r="O211" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
         <v/>
       </c>
       <c r="D213" s="2" t="n">
-        <v>184.4957514859501</v>
+        <v>184.4957514859502</v>
       </c>
       <c r="E213" s="2" t="n">
         <v>0</v>
@@ -11735,10 +11735,10 @@
         <v>0</v>
       </c>
       <c r="H213" s="2" t="n">
-        <v>39.44206538482189</v>
+        <v>39.44206538518096</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>10.05297497521063</v>
+        <v>10.05297501303865</v>
       </c>
       <c r="J213" s="2" t="n">
         <v>0</v>
@@ -11753,7 +11753,7 @@
         <v>-1</v>
       </c>
       <c r="N213" s="2" t="n">
-        <v>-2.646243447355126</v>
+        <v>-2.646243447562783</v>
       </c>
       <c r="O213" s="2" t="inlineStr">
         <is>
@@ -11880,7 +11880,7 @@
         <v/>
       </c>
       <c r="D216" s="2" t="n">
-        <v>178.3599327864884</v>
+        <v>178.3599327864889</v>
       </c>
       <c r="E216" s="2" t="n">
         <v>257</v>
@@ -11894,10 +11894,10 @@
         <v>0</v>
       </c>
       <c r="H216" s="2" t="n">
-        <v>32.01263934042265</v>
+        <v>32.01263952027533</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>19.43690846384547</v>
+        <v>19.4369086859546</v>
       </c>
       <c r="J216" s="2" t="n">
         <v>1.072517975781797</v>
@@ -11912,7 +11912,7 @@
         <v>-1</v>
       </c>
       <c r="N216" s="2" t="n">
-        <v>-2.060709038281889</v>
+        <v>-2.060709037113789</v>
       </c>
       <c r="O216" s="2" t="inlineStr">
         <is>
@@ -12053,10 +12053,10 @@
         <v>0</v>
       </c>
       <c r="H219" s="2" t="n">
-        <v>39.3687339859857</v>
+        <v>39.36873373239074</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>17.14593224613341</v>
+        <v>17.14593208750387</v>
       </c>
       <c r="J219" s="2" t="n">
         <v>0.5796078806754489</v>
@@ -12071,7 +12071,7 @@
         <v>-1</v>
       </c>
       <c r="N219" s="2" t="n">
-        <v>-0.03442011168482986</v>
+        <v>-0.03442011154206354</v>
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
@@ -12145,7 +12145,7 @@
         <v/>
       </c>
       <c r="D221" s="2" t="n">
-        <v>164.9222530648884</v>
+        <v>164.9222530648883</v>
       </c>
       <c r="E221" s="2" t="n">
         <v>80.2</v>
@@ -12159,10 +12159,10 @@
         <v>0</v>
       </c>
       <c r="H221" s="2" t="n">
-        <v>41.06497063247135</v>
+        <v>41.06497055785508</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>18.49328749843953</v>
+        <v>18.49328741484167</v>
       </c>
       <c r="J221" s="2" t="n">
         <v>0.7394850716562866</v>
@@ -12177,7 +12177,7 @@
         <v>-1</v>
       </c>
       <c r="N221" s="2" t="n">
-        <v>-0.6563706099980144</v>
+        <v>-0.6563706094788744</v>
       </c>
       <c r="O221" s="2" t="inlineStr">
         <is>
@@ -12251,7 +12251,7 @@
         <v/>
       </c>
       <c r="D223" s="2" t="n">
-        <v>149.4953231177808</v>
+        <v>149.4953231177823</v>
       </c>
       <c r="E223" s="2" t="n">
         <v>15.3</v>
@@ -12265,10 +12265,10 @@
         <v>0</v>
       </c>
       <c r="H223" s="2" t="n">
-        <v>26.89006021069351</v>
+        <v>26.89006023579327</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>9.232916954990296</v>
+        <v>9.232916954990298</v>
       </c>
       <c r="J223" s="2" t="n">
         <v>0.4547855288837673</v>
@@ -12283,7 +12283,7 @@
         <v>-1</v>
       </c>
       <c r="N223" s="2" t="n">
-        <v>-0.03382831797910943</v>
+        <v>-0.03382831799208827</v>
       </c>
       <c r="O223" s="2" t="inlineStr">
         <is>
@@ -12318,10 +12318,10 @@
         <v>0</v>
       </c>
       <c r="H224" s="2" t="n">
-        <v>23.08692412285592</v>
+        <v>23.08692435527524</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>34.15634869585315</v>
+        <v>34.15634874110015</v>
       </c>
       <c r="J224" s="2" t="n">
         <v>0.4444148041289535</v>
@@ -12336,7 +12336,7 @@
         <v>-1</v>
       </c>
       <c r="N224" s="2" t="n">
-        <v>-0.04030716898690179</v>
+        <v>-0.04030716909073584</v>
       </c>
       <c r="O224" s="2" t="inlineStr">
         <is>
@@ -12357,7 +12357,7 @@
         <v/>
       </c>
       <c r="D225" s="2" t="n">
-        <v>140.9441167265884</v>
+        <v>140.9441167265883</v>
       </c>
       <c r="E225" s="2" t="n">
         <v>180.5</v>
@@ -12371,10 +12371,10 @@
         <v>0</v>
       </c>
       <c r="H225" s="2" t="n">
-        <v>41.92679828073859</v>
+        <v>41.92679836243252</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>16.12154018558874</v>
+        <v>16.12154025081828</v>
       </c>
       <c r="J225" s="2" t="n">
         <v>0.2417078986138679</v>
@@ -12389,7 +12389,7 @@
         <v>-1</v>
       </c>
       <c r="N225" s="2" t="n">
-        <v>-0.4932059135302538</v>
+        <v>-0.4932059141791543</v>
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
@@ -12463,7 +12463,7 @@
         <v/>
       </c>
       <c r="D227" s="2" t="n">
-        <v>134.078144386023</v>
+        <v>134.0781443860232</v>
       </c>
       <c r="E227" s="2" t="n">
         <v>49.4</v>
@@ -12477,10 +12477,10 @@
         <v>0</v>
       </c>
       <c r="H227" s="2" t="n">
-        <v>38.7876893853287</v>
+        <v>38.78768942745078</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>14.83387708121921</v>
+        <v>14.83387717016408</v>
       </c>
       <c r="J227" s="2" t="n">
         <v>1.322178151095284</v>
@@ -12495,7 +12495,7 @@
         <v>-1</v>
       </c>
       <c r="N227" s="2" t="n">
-        <v>-0.3395202393403831</v>
+        <v>-0.3395202393922944</v>
       </c>
       <c r="O227" s="2" t="inlineStr">
         <is>
@@ -12689,7 +12689,7 @@
         <v>0</v>
       </c>
       <c r="H231" s="2" t="n">
-        <v>40.55479290861305</v>
+        <v>40.55479302872619</v>
       </c>
       <c r="I231" s="2" t="n">
         <v>13.64055444355624</v>
@@ -12707,7 +12707,7 @@
         <v>-1</v>
       </c>
       <c r="N231" s="2" t="n">
-        <v>-0.1265280396838262</v>
+        <v>-0.1265280396578688</v>
       </c>
       <c r="O231" s="2" t="inlineStr">
         <is>
@@ -12904,7 +12904,7 @@
         <v>34.81277821155926</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>10.74313231419725</v>
+        <v>10.74313229007495</v>
       </c>
       <c r="J235" s="2" t="n">
         <v>1.088511274073588</v>
@@ -12940,7 +12940,7 @@
         <v/>
       </c>
       <c r="D236" s="2" t="n">
-        <v>80.58502275337251</v>
+        <v>80.58502275337247</v>
       </c>
       <c r="E236" s="2" t="n">
         <v>47</v>
@@ -12954,10 +12954,10 @@
         <v>0</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>39.53376049133681</v>
+        <v>39.53376070501145</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>12.92250409757598</v>
+        <v>12.92250427398179</v>
       </c>
       <c r="J236" s="2" t="n">
         <v>0.6961502402437595</v>
@@ -12972,7 +12972,7 @@
         <v>-1</v>
       </c>
       <c r="N236" s="2" t="n">
-        <v>-0.2426595612904388</v>
+        <v>-0.2426595620691573</v>
       </c>
       <c r="O236" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg4 2026-10-27 00:09 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq5_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>58.71540732949924</v>
+        <v>58.71540734635067</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>31.50463002584766</v>
+        <v>31.50463023168091</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.187862502101565</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.219326619872409</v>
+        <v>0.2193266195640363</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>60.36293115425422</v>
+        <v>60.36293118891671</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>17.80203770417078</v>
+        <v>17.80203772167448</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>6.471057182710961</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.03785613179024211</v>
+        <v>0.03785613174819033</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>81.94581891383891</v>
+        <v>81.94581891130534</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>49.98489027130555</v>
+        <v>49.98489021057809</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>3.27165641082714</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.5022326844181748</v>
+        <v>0.5022326844462084</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>57.21533962858903</v>
+        <v>57.21533965458255</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>23.01003657029381</v>
+        <v>23.01003669951026</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.6538297063575026</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>-0.006386105262095043</v>
+        <v>-0.006386105822778987</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>67.47730871564642</v>
+        <v>67.47730871288752</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>38.50702402157852</v>
+        <v>38.50702399073548</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.7091061402198082</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.111542975803565</v>
+        <v>1.111542975831595</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65.72648825626538</v>
+        <v>65.72648919232421</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>36.53375580982868</v>
+        <v>36.5337581107967</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.692503306164643</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.8017789735967824</v>
+        <v>0.8017789689151087</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>73.72072187995276</v>
+        <v>73.72072183951929</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>31.74214433322286</v>
+        <v>31.74214435630711</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.8762501428629438</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.7024521164294275</v>
+        <v>0.7024521165415629</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>80.35938204487961</v>
+        <v>80.35938202261842</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>39.79969103353677</v>
+        <v>39.79969126080731</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>5.11066440824874</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.7807430087987781</v>
+        <v>0.7807430088127938</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>81.88737139791144</v>
+        <v>81.88737147549216</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>36.07106731354176</v>
+        <v>36.07106760404669</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.462659166782096</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>3.361381663639384</v>
+        <v>3.361381662812383</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62.97480634881731</v>
+        <v>62.9748062866202</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>24.69193176386295</v>
+        <v>24.69193177451364</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.158462452084048</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>55.81706509751536</v>
+        <v>55.81706513075596</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>32.32710441045417</v>
+        <v>32.32710436662455</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.787900186130918</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.1276567221524842</v>
+        <v>0.1276567220683782</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>53.27529813927573</v>
+        <v>53.2752980933955</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>25.60942187399197</v>
+        <v>25.60942189840431</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.8154616570838</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.08295403207349317</v>
+        <v>-0.08295403193333817</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>63.02984614055978</v>
+        <v>63.02984631528551</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>21.0621366495543</v>
+        <v>21.06213660525024</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>6.428143915657802</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.3145315477401854</v>
+        <v>0.3145315473757477</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>55.90932651088788</v>
+        <v>55.9093265721194</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>31.04182783555339</v>
+        <v>31.04182790598966</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>2.110484204362749</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>-0.03059697940867989</v>
+        <v>-0.03059697945073037</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>56.7433131420784</v>
+        <v>56.74331316723455</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>21.01212501621335</v>
+        <v>21.01212502683116</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>1.31062325989884</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.6810293733526969</v>
+        <v>-0.6810293751748233</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>742.2968497228387</v>
+        <v>742.2968497228386</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>67.40000000000001</v>
@@ -1774,7 +1774,7 @@
         <v>57.09436543969906</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>45.20271233297377</v>
+        <v>45.20271238393471</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.4002431834369567</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>83.69258322527864</v>
+        <v>83.6925832740047</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>45.70492444448431</v>
+        <v>45.70492472214745</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.454910189928036</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.6535139426709955</v>
+        <v>0.6535139426009133</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>67.1037655016944</v>
+        <v>67.10376545776759</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>32.15298274396929</v>
+        <v>32.15298270512947</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.227640664266034</v>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>53.71904253191844</v>
+        <v>53.71904261690501</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>37.25047813442104</v>
+        <v>37.25047808605032</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>1.808486933152997</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.2087696313257501</v>
+        <v>0.2087696305688302</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.45873626539827</v>
+        <v>54.45873632903957</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>45.04771733600305</v>
+        <v>45.04771738936108</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.6020709366803771</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-0.1109833868284922</v>
+        <v>-0.1109833868845596</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>56.78185576895208</v>
+        <v>56.78185576794199</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>41.77704599464007</v>
+        <v>41.77704601690757</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.4664102457209825</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.1153225829105862</v>
+        <v>-0.1153225828909636</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>44.5264246905391</v>
+        <v>44.52642469727785</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>24.53325134070302</v>
+        <v>24.53325131449401</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.3576261418734671</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-1.224199263591962</v>
+        <v>-1.224199263339663</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>54.87024429186362</v>
+        <v>54.87024430593537</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>23.73600204318079</v>
+        <v>23.73600203460547</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.744313648013688</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.8343936670345076</v>
+        <v>0.8343936666980916</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>643.0286015091606</v>
+        <v>643.0286015091687</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>24.15</v>
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>58.45871392402407</v>
+        <v>58.45871378785053</v>
       </c>
       <c r="I35" s="2" t="n">
         <v>11.62867272595374</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.07830300175994642</v>
+        <v>0.07830300192815122</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>53.07434670598008</v>
+        <v>53.07434690979996</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>41.47306182264293</v>
+        <v>41.47306202501695</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.9546270210683551</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.1560608191991033</v>
+        <v>0.1560608186944861</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>59.59249117982401</v>
+        <v>59.59249118217048</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20.32430295801651</v>
+        <v>20.32430298663114</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>2.747844849271973</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.2480613860502487</v>
+        <v>0.2480613854475098</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>50.82841791275604</v>
+        <v>50.8284179527244</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>20.95883844924494</v>
+        <v>20.95883846525075</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>2.111377077425062</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>1.05963939555556</v>
+        <v>1.059639395373346</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>44.25004963421338</v>
+        <v>44.25004965413164</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>25.3285408351281</v>
+        <v>25.32854096584945</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.1645504737079533</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.8458468375653205</v>
+        <v>-0.8458468376354065</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>50.75643636564652</v>
+        <v>50.75643656268497</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>28.22583981681614</v>
+        <v>28.22584004555938</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.2665126809855208</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.07269387127574053</v>
+        <v>-0.07269387141987799</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>618.6030927328005</v>
+        <v>618.6030927328006</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>93.59999999999999</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>49.22334189141193</v>
+        <v>49.22334204080315</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>21.00094103024897</v>
+        <v>21.00094117981484</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.8802939404741535</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.3038884513579403</v>
+        <v>-0.3038884523391248</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>615.4214150174516</v>
+        <v>615.4214150174519</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>188.5</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>57.09404385677026</v>
+        <v>57.09404383564659</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>38.03058888987331</v>
+        <v>38.03058903982319</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.5408367626420775</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.4235338442664052</v>
+        <v>-0.4235338449672525</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>593.1013509456421</v>
+        <v>593.1013509456275</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>17.1</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>53.77654893270888</v>
+        <v>53.77654904065064</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>31.72330381001659</v>
+        <v>31.72330435521455</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.6789348499202551</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.005243950350679163</v>
+        <v>0.005243950995460961</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>584.880022806052</v>
+        <v>584.8800228060517</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>81.59999999999999</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>55.06320498775857</v>
+        <v>55.06283778103794</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>23.9084010100203</v>
+        <v>23.90861557192525</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.750864911342356</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.04088320773392098</v>
+        <v>-0.04088281629673879</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>53.94389996875152</v>
+        <v>53.9439000261244</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>44.27465337150566</v>
+        <v>44.27465339088047</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5584352714811873</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.02812732035400733</v>
+        <v>0.02812732004564245</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>50.77997812813894</v>
+        <v>50.77997813095823</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>30.19243493941238</v>
+        <v>30.19243503839056</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.6311428437812682</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.1829075867058967</v>
+        <v>-0.1829075866358094</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>47.83022559106772</v>
+        <v>47.83022559866096</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>37.85256857113046</v>
+        <v>37.85256861726808</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>1.1802974941166</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.1213752903850946</v>
+        <v>-0.1213752904551808</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3029,7 +3029,7 @@
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>557.1688015126584</v>
+        <v>557.1688015126585</v>
       </c>
       <c r="E49" s="2" t="n">
         <v>17.75</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>48.69244694482845</v>
+        <v>48.69244701273587</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>24.75134292688713</v>
+        <v>24.75134305415404</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1.010074009411962</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.01503209315566223</v>
+        <v>0.01503209307156084</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>56.11600236935473</v>
+        <v>56.11600240559136</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>53.09777368739398</v>
+        <v>53.097773894124</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.6728282127834375</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.23034833728912</v>
+        <v>-0.2303483374993784</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>44.94157558209933</v>
+        <v>44.94157557116918</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>35.76088523194549</v>
+        <v>35.76088527068059</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.4702770291925662</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1317302112378655</v>
+        <v>-0.1317302112406689</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.17923266758795</v>
+        <v>49.17923282717558</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.08847688687782</v>
+        <v>22.08847692941036</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.676634979807586</v>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>543.1860384189425</v>
+        <v>543.1860384189428</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>66</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>50.46380263036743</v>
+        <v>50.4638026202951</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>35.33190735487626</v>
+        <v>35.33190735809912</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.3482522570893783</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-0.06957806434704361</v>
+        <v>-0.06957806440309922</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>40.18949045887918</v>
+        <v>40.1894905285012</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>17.3784076482947</v>
+        <v>17.37840761612043</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.9249136326467248</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.2580446862705221</v>
+        <v>0.2580446841680635</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>535.3845042756371</v>
+        <v>535.3845042756367</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>99.59999999999999</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>46.63044490121426</v>
+        <v>46.63044512453518</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>22.01828716164973</v>
+        <v>22.01828729624412</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.8275487601044539</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.2624983392130469</v>
+        <v>-0.2624983397456871</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>514.6867921553664</v>
+        <v>514.6867921553666</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>36.65</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>53.12262155453313</v>
+        <v>53.1226216694909</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>32.60868648626341</v>
+        <v>32.60868653145738</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.1586045019890487</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-0.26872811296396</v>
+        <v>-0.2687281130901098</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>43.67270683903508</v>
+        <v>43.67270684863689</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>24.01465263890841</v>
+        <v>24.01465281576952</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.546138966227986</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-5.474442633609591</v>
+        <v>-5.474442634310428</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>53.11887040934334</v>
+        <v>53.11887049975827</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>48.90186894664097</v>
+        <v>48.90186930154012</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3428531919249178</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.06435409286212113</v>
+        <v>-0.06435409297425632</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>49.82525829136053</v>
+        <v>49.82525835819582</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>25.41803893714081</v>
+        <v>25.41803901897512</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.6805115273915329</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.3366953822198397</v>
+        <v>-0.3366953823319748</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3894,7 +3894,7 @@
         <v>50.16229171528452</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>6.246335708498706</v>
+        <v>6.246335640274697</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.874878600138947</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>42.90798957595698</v>
+        <v>42.90798956736265</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>23.90486651606784</v>
+        <v>23.90486654747815</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.3668306422469273</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-3.022196359113328</v>
+        <v>-3.022196359057276</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>48.35028336370146</v>
+        <v>48.3502834796975</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>17.62947805580007</v>
+        <v>17.62947812232312</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.9233897323927502</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-5.226016157073865</v>
+        <v>-5.226016158475673</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>481.3892436431061</v>
+        <v>481.3892436431062</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>18.6</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.90797382230961</v>
+        <v>42.90797319071532</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>26.16036450602836</v>
+        <v>26.16036470523188</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.608415001976404</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.02362445722941669</v>
+        <v>-0.02362445685095621</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.54773018107319</v>
+        <v>46.54773021323055</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>35.54764260221483</v>
+        <v>35.54764261993768</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.8080786915686315</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.02472815294493658</v>
+        <v>-0.02472815169742448</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>50.7500966296235</v>
+        <v>50.75009666486213</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>29.20609822816496</v>
+        <v>29.20609825338403</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.9061301977907532</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-3.08760260292868</v>
+        <v>-3.087602603909822</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>466.4285035895276</v>
+        <v>466.4285035895273</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>291.5</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>44.19423805601657</v>
+        <v>44.19423829204025</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>19.80632466485373</v>
+        <v>19.80632464683062</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.4447717766434362</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-2.301545053070018</v>
+        <v>-2.30154505391101</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>42.89302857351618</v>
+        <v>42.89302862041029</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>21.26840078660977</v>
+        <v>21.26840085797989</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.6030305606881261</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-3.134957997143606</v>
+        <v>-3.134957997564108</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>459.5345957077824</v>
+        <v>459.5345957077823</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>14.6</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>47.2161360732695</v>
+        <v>47.21613643133246</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>25.60402402105941</v>
+        <v>25.60402432029144</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.6202603567782652</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0006856950873350715</v>
+        <v>-0.0006856952695538186</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>454.9208084580182</v>
+        <v>454.9208084580185</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>345</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>52.02037517621718</v>
+        <v>52.02037517132116</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>31.18402020979075</v>
+        <v>31.18402024259196</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>1.180801934696807</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.5544916651847061</v>
+        <v>0.5544916652408034</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>60.0249746630809</v>
+        <v>60.02497464919667</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>35.68442775405224</v>
+        <v>35.68442789396749</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.6708265725262842</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.1625535905192448</v>
+        <v>0.1625535905612951</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>448.7307920607386</v>
+        <v>448.7307920607387</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>13.65</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>49.61056875233533</v>
+        <v>49.61056884089233</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>29.06409289683194</v>
+        <v>29.06409288143472</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.1924478965139438</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.01490187012695563</v>
+        <v>-0.01490187022507428</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>447.1863521922413</v>
+        <v>447.1863521922414</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>62</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.40573270723296</v>
+        <v>43.40573281996762</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>20.97532759183924</v>
+        <v>20.97532749842548</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>1.339903640251592</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.3008378259612848</v>
+        <v>-0.3008378259893116</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>35.8085511964649</v>
+        <v>35.80855124376482</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>17.15925860607282</v>
+        <v>17.15925860998989</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.6246090928836558</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-2.231573269123184</v>
+        <v>-2.231573269683839</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.06128102015975</v>
+        <v>49.06128099342555</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>16.54223314078174</v>
+        <v>16.54223321834086</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.3477868282759332</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.291361405602417</v>
+        <v>-0.2913614057005385</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>56.30428731737776</v>
+        <v>56.3042873105371</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>26.83748183858352</v>
+        <v>26.83748201088983</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.392288391984023</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.2875674543305244</v>
+        <v>-0.2875674542604467</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>434.6857687521248</v>
+        <v>434.6857687521249</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>17.3</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>31.85403095620745</v>
+        <v>31.85403106164044</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>37.78841225050679</v>
+        <v>37.78841259543034</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.918010049699698</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.01017590790040424</v>
+        <v>-0.01017590794245671</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>44.96759671932401</v>
+        <v>44.96759671035566</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>30.32974215634031</v>
+        <v>30.32974222770279</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.3184646564163551</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.1281383475446506</v>
+        <v>-0.128138347572685</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>49.66570543835159</v>
+        <v>49.66570597900246</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>22.42465627205382</v>
+        <v>22.42465627205381</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.3145166128189087</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.00136020170098182</v>
+        <v>0.001360201098256991</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>40.4228123873171</v>
+        <v>40.42281240888585</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>13.54499931694578</v>
+        <v>13.54499943623492</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.6523495815408242</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.185893966387279</v>
+        <v>-1.185893966583511</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>416.7405722250556</v>
+        <v>416.7405722250555</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>450</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>34.87559539522162</v>
+        <v>34.8755954103069</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>16.96497705809955</v>
+        <v>16.96497707582093</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.6578222675025817</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-13.24911078760191</v>
+        <v>-13.24911078970446</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>416.2566732293046</v>
+        <v>416.2566732293049</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>450</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>36.51115250253315</v>
+        <v>36.51115252903333</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>16.64076263252731</v>
+        <v>16.64076283297378</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.2296701478970592</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-13.63130627464767</v>
+        <v>-13.63130627520836</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>413.840623182328</v>
+        <v>413.8406231823279</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>415</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>39.09931713986931</v>
+        <v>39.09931711059583</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>11.58223399364486</v>
+        <v>11.58223401929437</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.6426868025653274</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-8.233670896876708</v>
+        <v>-8.233670896596335</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>51.47993822080375</v>
+        <v>51.47993827319218</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>24.67226676830401</v>
+        <v>24.67226681355426</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>1.07424450654123</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>33.25653630160207</v>
+        <v>33.25653630400232</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>27.40786541420307</v>
+        <v>27.40786540610959</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.2688001915480837</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-1.767537340207883</v>
+        <v>-1.76753734027797</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5749,7 +5749,7 @@
         <v>48.96009149685735</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>24.57627482011732</v>
+        <v>24.57627475437191</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.3522834717951072</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>32.59205737992454</v>
+        <v>32.59205745710064</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>22.33610688919616</v>
+        <v>22.33610697713728</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.4706526780345856</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-4.284881463491689</v>
+        <v>-4.284881466154917</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>388.1162917329289</v>
+        <v>388.116291732929</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>43.8</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>47.72205062719986</v>
+        <v>47.72205069016473</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>26.85301736203532</v>
+        <v>26.85301740298347</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.7756948546847828</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>0.3016156866558141</v>
+        <v>0.3016156865717119</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>41.26720461186287</v>
+        <v>41.26720470315009</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>18.25417885356874</v>
+        <v>18.25417887098569</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.5628364826975915</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-1.243661215827961</v>
+        <v>-1.243661215491553</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>34.10721353293057</v>
+        <v>34.10721346976806</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>22.60116772618948</v>
+        <v>22.60116783998096</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.4155596742635219</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-18.05247321939985</v>
+        <v>-18.05247323285609</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>375.4686592806291</v>
+        <v>375.4686592806285</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>40.1</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>40.75018685678466</v>
+        <v>40.75018702167016</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>24.45809747722878</v>
+        <v>24.45809793441233</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.5398989861642104</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.1610759611141016</v>
+        <v>-0.161075961254272</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>40.00908295336473</v>
+        <v>40.00908303568576</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>19.24325222305583</v>
+        <v>19.24325229355994</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.3984613648528562</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-1.395478721712399</v>
+        <v>-1.395478721964701</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>369.5531730137181</v>
+        <v>369.553173013718</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>1065</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>26.66817974788805</v>
+        <v>26.66817975510037</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>22.66585688902772</v>
+        <v>22.66585696093522</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.9613527360345413</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-12.7121906466236</v>
+        <v>-12.71219064732438</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>34.55778175776258</v>
+        <v>34.5577817735042</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>16.24835060323948</v>
+        <v>16.24835073880199</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.4548212397948666</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.4405644328794132</v>
+        <v>-0.4405644329214644</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>45.82001236236686</v>
+        <v>45.82001245292849</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>23.88250129175117</v>
+        <v>23.88250138252617</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.7588529169742557</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.08853583840282894</v>
+        <v>-0.08853583848693058</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6421,7 @@
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>364.9939452106958</v>
+        <v>364.9939452106959</v>
       </c>
       <c r="E113" s="2" t="n">
         <v>132.5</v>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>39.89940563797986</v>
+        <v>39.89940564651337</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>16.8364344252073</v>
+        <v>16.83643445938989</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.6176754398396934</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.6923510208442794</v>
+        <v>-0.6923510208863318</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>364.2427140738569</v>
+        <v>364.2427140738566</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>165</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>44.6809220759878</v>
+        <v>44.68092212150973</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>25.40918254008711</v>
+        <v>25.40918265199017</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.8533687089202689</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-1.355937889045877</v>
+        <v>-1.355937889466373</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.30845755382955</v>
+        <v>47.30845759171962</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>27.00294437244895</v>
+        <v>27.00294437640576</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.4161983283834993</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-2.225607502938787</v>
+        <v>-2.225607503022889</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>361.7225533573798</v>
+        <v>361.7225533573799</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>85.5</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>36.7363317664434</v>
+        <v>36.73633190316522</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>29.7257038889804</v>
+        <v>29.7257038883947</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.8360942421390062</v>
@@ -6739,7 +6739,7 @@
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>360.7744839129663</v>
+        <v>360.7744839129667</v>
       </c>
       <c r="E119" s="2" t="n">
         <v>27.7</v>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>41.80378248029942</v>
+        <v>41.80378249858325</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>24.25112712583495</v>
+        <v>24.25112720699056</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.4769226661557043</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.1174176892371887</v>
+        <v>-0.1174176892231732</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>358.1433075754225</v>
+        <v>358.1433075754226</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>16010</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>39.50698521585365</v>
+        <v>39.50698525583839</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.6985730124443</v>
+        <v>18.69857317722544</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.8402950493068254</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-308.7511184109266</v>
+        <v>-308.7511184613871</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>46.30494914905276</v>
+        <v>46.304949314849</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>15.48152845522575</v>
+        <v>15.48152847851205</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.3015382345052691</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.23046324667413</v>
+        <v>-0.230463246954472</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>49.82068965804196</v>
+        <v>49.82069925959484</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>19.28851097007136</v>
+        <v>19.2885166377338</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.2246838673564136</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.1359219512694098</v>
+        <v>-0.1359219570864572</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>29.767389403103</v>
+        <v>29.76738940655838</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>36.31166146959956</v>
+        <v>36.31166149394019</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.7975547534955224</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-3.080267690219187</v>
+        <v>-3.080267690331336</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>30.56645086747565</v>
+        <v>30.56645087873255</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>21.13261890627402</v>
+        <v>21.13261877461661</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>1.435301620678291</v>
@@ -7534,7 +7534,7 @@
         <v/>
       </c>
       <c r="D134" s="2" t="n">
-        <v>329.5075426442443</v>
+        <v>329.5075426442444</v>
       </c>
       <c r="E134" s="2" t="n">
         <v>16.25</v>
@@ -7548,10 +7548,10 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>51.22298547319819</v>
+        <v>51.22298531483361</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>29.92738464253872</v>
+        <v>29.9273846480226</v>
       </c>
       <c r="J134" s="2" t="n">
         <v>0.4245008099934375</v>
@@ -7566,7 +7566,7 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>0.01632932260729233</v>
+        <v>0.0163293226353249</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
@@ -7640,7 +7640,7 @@
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>323.9660901587906</v>
+        <v>323.9660901587908</v>
       </c>
       <c r="E136" s="2" t="n">
         <v>99.40000000000001</v>
@@ -7654,10 +7654,10 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>37.51994403480123</v>
+        <v>37.51994406674557</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>20.16741347046085</v>
+        <v>20.16741346935512</v>
       </c>
       <c r="J136" s="2" t="n">
         <v>0.7410247126840072</v>
@@ -7672,7 +7672,7 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-1.456166476743258</v>
+        <v>-1.45616647665915</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
@@ -7760,10 +7760,10 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>43.89240197374205</v>
+        <v>43.89240201433005</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>16.69250958176906</v>
+        <v>16.6925094991455</v>
       </c>
       <c r="J138" s="2" t="n">
         <v>0.7467043119600456</v>
@@ -7799,7 +7799,7 @@
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>317.2554041227373</v>
+        <v>317.2554041227372</v>
       </c>
       <c r="E139" s="2" t="n">
         <v>25.1</v>
@@ -7813,10 +7813,10 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>39.05537920710675</v>
+        <v>39.05537953693277</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>12.35170998657356</v>
+        <v>12.3517100038439</v>
       </c>
       <c r="J139" s="2" t="n">
         <v>0.8868180782148205</v>
@@ -7831,7 +7831,7 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>0.2626710628691629</v>
+        <v>0.2626710635700134</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
@@ -7919,10 +7919,10 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>49.0599712826354</v>
+        <v>49.05997646263963</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>19.84839471967957</v>
+        <v>19.84839413371592</v>
       </c>
       <c r="J141" s="2" t="n">
         <v>0.1790799411206339</v>
@@ -7937,7 +7937,7 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>-0.1002585730876456</v>
+        <v>-0.1002585599327223</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
@@ -7958,7 +7958,7 @@
         <v/>
       </c>
       <c r="D142" s="2" t="n">
-        <v>313.1024174236519</v>
+        <v>313.102417423653</v>
       </c>
       <c r="E142" s="2" t="n">
         <v>21.5</v>
@@ -7972,10 +7972,10 @@
         <v>0</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>41.7095473525884</v>
+        <v>41.70954755102171</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>28.80249823788058</v>
+        <v>28.80249824429122</v>
       </c>
       <c r="J142" s="2" t="n">
         <v>0.6564208576689142</v>
@@ -7990,7 +7990,7 @@
         <v>-1</v>
       </c>
       <c r="N142" s="2" t="n">
-        <v>-0.02910323438228091</v>
+        <v>-0.02910323453798225</v>
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
@@ -8025,10 +8025,10 @@
         <v>0</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>42.37594703200608</v>
+        <v>42.37594744434298</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>23.06708923031829</v>
+        <v>23.06708952173175</v>
       </c>
       <c r="J143" s="2" t="n">
         <v>0.5290952715368873</v>
@@ -8043,7 +8043,7 @@
         <v>-1</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>-0.009005245303026849</v>
+        <v>-0.009005245415167784</v>
       </c>
       <c r="O143" s="2" t="inlineStr">
         <is>
@@ -8064,7 +8064,7 @@
         <v/>
       </c>
       <c r="D144" s="2" t="n">
-        <v>307.3501794806456</v>
+        <v>307.3501794806439</v>
       </c>
       <c r="E144" s="2" t="n">
         <v>15.45</v>
@@ -8078,10 +8078,10 @@
         <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>42.43231215763032</v>
+        <v>42.43231298979521</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>26.75579892174356</v>
+        <v>26.75579929531296</v>
       </c>
       <c r="J144" s="2" t="n">
         <v>0.2826159701525211</v>
@@ -8096,7 +8096,7 @@
         <v>-1</v>
       </c>
       <c r="N144" s="2" t="n">
-        <v>-0.07682118533193466</v>
+        <v>-0.07682118565432502</v>
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         <v/>
       </c>
       <c r="D145" s="2" t="n">
-        <v>307.1737837360084</v>
+        <v>307.173783736008</v>
       </c>
       <c r="E145" s="2" t="n">
         <v>640</v>
@@ -8131,10 +8131,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>31.34850298967814</v>
+        <v>31.3485030419905</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>26.95158512503191</v>
+        <v>26.95158511633877</v>
       </c>
       <c r="J145" s="2" t="n">
         <v>0.5634934586368862</v>
@@ -8149,7 +8149,7 @@
         <v>-1</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>-11.78792777952359</v>
+        <v>-11.78792778274748</v>
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8329,7 +8329,7 @@
         <v/>
       </c>
       <c r="D149" s="2" t="n">
-        <v>302.4465644582874</v>
+        <v>302.4465644582875</v>
       </c>
       <c r="E149" s="2" t="n">
         <v>8.710000000000001</v>
@@ -8343,10 +8343,10 @@
         <v>0</v>
       </c>
       <c r="H149" s="2" t="n">
-        <v>40.37581441761522</v>
+        <v>40.37581334478844</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>31.91115574505688</v>
+        <v>31.91115573554907</v>
       </c>
       <c r="J149" s="2" t="n">
         <v>1.391582627497993</v>
@@ -8361,7 +8361,7 @@
         <v>-1</v>
       </c>
       <c r="N149" s="2" t="n">
-        <v>-0.03246650582306902</v>
+        <v>-0.03246650539599838</v>
       </c>
       <c r="O149" s="2" t="inlineStr">
         <is>
@@ -8396,10 +8396,10 @@
         <v>0</v>
       </c>
       <c r="H150" s="2" t="n">
-        <v>45.03272834660827</v>
+        <v>45.03272837795529</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>12.96847207881039</v>
+        <v>12.96847213424285</v>
       </c>
       <c r="J150" s="2" t="n">
         <v>1.295965100731432</v>
@@ -8414,7 +8414,7 @@
         <v>-1</v>
       </c>
       <c r="N150" s="2" t="n">
-        <v>-0.3285368726226759</v>
+        <v>-0.3285368727628438</v>
       </c>
       <c r="O150" s="2" t="inlineStr">
         <is>
@@ -8661,10 +8661,10 @@
         <v>0</v>
       </c>
       <c r="H155" s="2" t="n">
-        <v>42.42086002303296</v>
+        <v>42.4208600542883</v>
       </c>
       <c r="I155" s="2" t="n">
-        <v>21.20655716716618</v>
+        <v>21.20655719330736</v>
       </c>
       <c r="J155" s="2" t="n">
         <v>0.7824611618735552</v>
@@ -8714,10 +8714,10 @@
         <v>0</v>
       </c>
       <c r="H156" s="2" t="n">
-        <v>42.2171398175153</v>
+        <v>42.21713984603075</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>19.86971297900487</v>
+        <v>19.8697131556773</v>
       </c>
       <c r="J156" s="2" t="n">
         <v>0.6065678297893753</v>
@@ -8732,7 +8732,7 @@
         <v>-1</v>
       </c>
       <c r="N156" s="2" t="n">
-        <v>-4.474363788063938</v>
+        <v>-4.47436378859657</v>
       </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
@@ -8767,10 +8767,10 @@
         <v>0</v>
       </c>
       <c r="H157" s="2" t="n">
-        <v>41.6076909167335</v>
+        <v>41.60769120165968</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>16.04394396519215</v>
+        <v>16.04394398385639</v>
       </c>
       <c r="J157" s="2" t="n">
         <v>0.8724937211523276</v>
@@ -8859,7 +8859,7 @@
         <v/>
       </c>
       <c r="D159" s="2" t="n">
-        <v>293.1465752264428</v>
+        <v>293.1465752264427</v>
       </c>
       <c r="E159" s="2" t="n">
         <v>67.7</v>
@@ -8873,10 +8873,10 @@
         <v>0</v>
       </c>
       <c r="H159" s="2" t="n">
-        <v>36.97738491281996</v>
+        <v>36.97738525266892</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>13.25062234785201</v>
+        <v>13.25062225152175</v>
       </c>
       <c r="J159" s="2" t="n">
         <v>1.876696144299828</v>
@@ -8891,7 +8891,7 @@
         <v>-1</v>
       </c>
       <c r="N159" s="2" t="n">
-        <v>-0.2258747490211306</v>
+        <v>-0.2258747493014777</v>
       </c>
       <c r="O159" s="2" t="inlineStr">
         <is>
@@ -8926,10 +8926,10 @@
         <v>0</v>
       </c>
       <c r="H160" s="2" t="n">
-        <v>49.06979965082504</v>
+        <v>49.06980173260322</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>7.760411504823782</v>
+        <v>7.760412919298332</v>
       </c>
       <c r="J160" s="2" t="n">
         <v>0.2019538779740827</v>
@@ -8944,7 +8944,7 @@
         <v>-1</v>
       </c>
       <c r="N160" s="2" t="n">
-        <v>0.03615697605028348</v>
+        <v>0.03615697007904842</v>
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
@@ -9018,7 +9018,7 @@
         <v/>
       </c>
       <c r="D162" s="2" t="n">
-        <v>290.8317395776794</v>
+        <v>290.8317395776825</v>
       </c>
       <c r="E162" s="2" t="n">
         <v>19</v>
@@ -9032,10 +9032,10 @@
         <v>0</v>
       </c>
       <c r="H162" s="2" t="n">
-        <v>45.47369756030899</v>
+        <v>45.47369805260906</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>22.03334029597098</v>
+        <v>22.03334038709632</v>
       </c>
       <c r="J162" s="2" t="n">
         <v>0.4876370636179536</v>
@@ -9050,7 +9050,7 @@
         <v>-1</v>
       </c>
       <c r="N162" s="2" t="n">
-        <v>-0.07910763639452899</v>
+        <v>-0.07910763674495262</v>
       </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
@@ -9244,10 +9244,10 @@
         <v>0</v>
       </c>
       <c r="H166" s="2" t="n">
-        <v>43.63312561331013</v>
+        <v>43.63312582823955</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>23.20104639580246</v>
+        <v>23.20104652913824</v>
       </c>
       <c r="J166" s="2" t="n">
         <v>0.3874471627102278</v>
@@ -9262,7 +9262,7 @@
         <v>-1</v>
       </c>
       <c r="N166" s="2" t="n">
-        <v>-0.3923335019888577</v>
+        <v>-0.3923335024374022</v>
       </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
@@ -9336,7 +9336,7 @@
         <v/>
       </c>
       <c r="D168" s="2" t="n">
-        <v>283.3204225637853</v>
+        <v>283.3204225637852</v>
       </c>
       <c r="E168" s="2" t="n">
         <v>14.75</v>
@@ -9350,10 +9350,10 @@
         <v>0</v>
       </c>
       <c r="H168" s="2" t="n">
-        <v>45.78300025013255</v>
+        <v>45.78300039969734</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>34.84264371061656</v>
+        <v>34.84264398904292</v>
       </c>
       <c r="J168" s="2" t="n">
         <v>0.6754960215755031</v>
@@ -9368,7 +9368,7 @@
         <v>-1</v>
       </c>
       <c r="N168" s="2" t="n">
-        <v>-0.1365065013050571</v>
+        <v>-0.1365065013471076</v>
       </c>
       <c r="O168" s="2" t="inlineStr">
         <is>
@@ -9442,7 +9442,7 @@
         <v/>
       </c>
       <c r="D170" s="2" t="n">
-        <v>275.636371846821</v>
+        <v>275.6363718468209</v>
       </c>
       <c r="E170" s="2" t="n">
         <v>83.5</v>
@@ -9456,10 +9456,10 @@
         <v>0</v>
       </c>
       <c r="H170" s="2" t="n">
-        <v>36.8892114444085</v>
+        <v>36.88921130259257</v>
       </c>
       <c r="I170" s="2" t="n">
-        <v>31.27097298692279</v>
+        <v>31.27097308149797</v>
       </c>
       <c r="J170" s="2" t="n">
         <v>0.4270185026716586</v>
@@ -9474,7 +9474,7 @@
         <v>-1</v>
       </c>
       <c r="N170" s="2" t="n">
-        <v>-1.021483902471753</v>
+        <v>-1.021483901995176</v>
       </c>
       <c r="O170" s="2" t="inlineStr">
         <is>
@@ -9615,10 +9615,10 @@
         <v>0</v>
       </c>
       <c r="H173" s="2" t="n">
-        <v>28.93627479253593</v>
+        <v>28.93627496983554</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>23.3046005625108</v>
+        <v>23.3046005643651</v>
       </c>
       <c r="J173" s="2" t="n">
         <v>2.374769044994032</v>
@@ -9654,7 +9654,7 @@
         <v/>
       </c>
       <c r="D174" s="2" t="n">
-        <v>269.2236864130882</v>
+        <v>269.2236864130892</v>
       </c>
       <c r="E174" s="2" t="n">
         <v>11.85</v>
@@ -9668,10 +9668,10 @@
         <v>0</v>
       </c>
       <c r="H174" s="2" t="n">
-        <v>48.45313078950023</v>
+        <v>48.45313082759859</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>10.8771229670505</v>
+        <v>10.87712298179298</v>
       </c>
       <c r="J174" s="2" t="n">
         <v>1.09492829634928</v>
@@ -9686,7 +9686,7 @@
         <v>-1</v>
       </c>
       <c r="N174" s="2" t="n">
-        <v>0.02334357571192497</v>
+        <v>0.02334357562782237</v>
       </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
@@ -9707,7 +9707,7 @@
         <v/>
       </c>
       <c r="D175" s="2" t="n">
-        <v>267.8002061668554</v>
+        <v>267.800206166855</v>
       </c>
       <c r="E175" s="2" t="n">
         <v>37</v>
@@ -9721,10 +9721,10 @@
         <v>0</v>
       </c>
       <c r="H175" s="2" t="n">
-        <v>38.10195546517012</v>
+        <v>38.10195553484263</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>23.7244578132024</v>
+        <v>23.7244578537106</v>
       </c>
       <c r="J175" s="2" t="n">
         <v>0.8299885544095317</v>
@@ -9739,7 +9739,7 @@
         <v>-1</v>
       </c>
       <c r="N175" s="2" t="n">
-        <v>0.02534579356034983</v>
+        <v>0.02534579326599307</v>
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>
@@ -9827,10 +9827,10 @@
         <v>0</v>
       </c>
       <c r="H177" s="2" t="n">
-        <v>34.90900996884839</v>
+        <v>34.90901008250478</v>
       </c>
       <c r="I177" s="2" t="n">
-        <v>24.36667189692079</v>
+        <v>24.36667182388068</v>
       </c>
       <c r="J177" s="2" t="n">
         <v>0.7401335990344164</v>
@@ -9845,7 +9845,7 @@
         <v>-1</v>
       </c>
       <c r="N177" s="2" t="n">
-        <v>-0.1010675392264537</v>
+        <v>-0.1010675396049114</v>
       </c>
       <c r="O177" s="2" t="inlineStr">
         <is>
@@ -9880,10 +9880,10 @@
         <v>0</v>
       </c>
       <c r="H178" s="2" t="n">
-        <v>50.98254581370494</v>
+        <v>50.98254533534474</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>12.88298332466061</v>
+        <v>12.8829833427588</v>
       </c>
       <c r="J178" s="2" t="n">
         <v>0.4696971423362655</v>
@@ -9898,7 +9898,7 @@
         <v>-1</v>
       </c>
       <c r="N178" s="2" t="n">
-        <v>-0.7577620943760697</v>
+        <v>-0.757762094305984</v>
       </c>
       <c r="O178" s="2" t="inlineStr">
         <is>
@@ -9972,7 +9972,7 @@
         <v/>
       </c>
       <c r="D180" s="2" t="n">
-        <v>259.6328817412765</v>
+        <v>259.6328817412755</v>
       </c>
       <c r="E180" s="2" t="n">
         <v>24.35</v>
@@ -9986,10 +9986,10 @@
         <v>0</v>
       </c>
       <c r="H180" s="2" t="n">
-        <v>50.8873066263123</v>
+        <v>50.88730666895655</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>14.54330288432353</v>
+        <v>14.54330294494826</v>
       </c>
       <c r="J180" s="2" t="n">
         <v>0.4030419221680238</v>
@@ -10004,7 +10004,7 @@
         <v>-1</v>
       </c>
       <c r="N180" s="2" t="n">
-        <v>0.3453550284224638</v>
+        <v>0.3453550283804112</v>
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
@@ -10092,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="H182" s="2" t="n">
-        <v>36.23390942518212</v>
+        <v>36.23391006332297</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>30.08902488147138</v>
+        <v>30.08902494216552</v>
       </c>
       <c r="J182" s="2" t="n">
         <v>0.9710557316499048</v>
@@ -10110,7 +10110,7 @@
         <v>-1</v>
       </c>
       <c r="N182" s="2" t="n">
-        <v>0.08411214670208866</v>
+        <v>0.08411214671610112</v>
       </c>
       <c r="O182" s="2" t="inlineStr">
         <is>
@@ -10145,10 +10145,10 @@
         <v>0</v>
       </c>
       <c r="H183" s="2" t="n">
-        <v>36.59352329362783</v>
+        <v>36.59352361954195</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>42.97112271220497</v>
+        <v>42.97112270803976</v>
       </c>
       <c r="J183" s="2" t="n">
         <v>0.8844312826620349</v>
@@ -10163,7 +10163,7 @@
         <v>-1</v>
       </c>
       <c r="N183" s="2" t="n">
-        <v>0.05722439603368346</v>
+        <v>0.05722439587949812</v>
       </c>
       <c r="O183" s="2" t="inlineStr">
         <is>
@@ -10184,7 +10184,7 @@
         <v/>
       </c>
       <c r="D184" s="2" t="n">
-        <v>252.6471212270199</v>
+        <v>252.6471212270202</v>
       </c>
       <c r="E184" s="2" t="n">
         <v>122</v>
@@ -10201,7 +10201,7 @@
         <v>32.35115412502192</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>29.52708789355588</v>
+        <v>29.52708790745055</v>
       </c>
       <c r="J184" s="2" t="n">
         <v>0.7964671735115098</v>
@@ -10216,7 +10216,7 @@
         <v>-1</v>
       </c>
       <c r="N184" s="2" t="n">
-        <v>-0.2649937664108259</v>
+        <v>-0.2649937661304849</v>
       </c>
       <c r="O184" s="2" t="inlineStr">
         <is>
@@ -10251,10 +10251,10 @@
         <v>0</v>
       </c>
       <c r="H185" s="2" t="n">
-        <v>23.20531902634664</v>
+        <v>23.20531904988853</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>28.1453719227303</v>
+        <v>28.14537192273031</v>
       </c>
       <c r="J185" s="2" t="n">
         <v>0.5590803840818684</v>
@@ -10269,7 +10269,7 @@
         <v>-1</v>
       </c>
       <c r="N185" s="2" t="n">
-        <v>-0.05160688986418438</v>
+        <v>-0.05160688990623608</v>
       </c>
       <c r="O185" s="2" t="inlineStr">
         <is>
@@ -10304,10 +10304,10 @@
         <v>0</v>
       </c>
       <c r="H186" s="2" t="n">
-        <v>34.93164446504781</v>
+        <v>34.93164457056116</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>20.90242728246207</v>
+        <v>20.90242748025634</v>
       </c>
       <c r="J186" s="2" t="n">
         <v>0.5188780721905544</v>
@@ -10322,7 +10322,7 @@
         <v>-1</v>
       </c>
       <c r="N186" s="2" t="n">
-        <v>-1.846751067500697</v>
+        <v>-1.846751069463075</v>
       </c>
       <c r="O186" s="2" t="inlineStr">
         <is>
@@ -10343,7 +10343,7 @@
         <v/>
       </c>
       <c r="D187" s="2" t="n">
-        <v>230.0041756847515</v>
+        <v>230.0041756847517</v>
       </c>
       <c r="E187" s="2" t="n">
         <v>17.05</v>
@@ -10357,10 +10357,10 @@
         <v>0</v>
       </c>
       <c r="H187" s="2" t="n">
-        <v>44.69491171625804</v>
+        <v>44.69491075583255</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>19.58619070519608</v>
+        <v>19.58619092221174</v>
       </c>
       <c r="J187" s="2" t="n">
         <v>0.6250509470229847</v>
@@ -10375,7 +10375,7 @@
         <v>-1</v>
       </c>
       <c r="N187" s="2" t="n">
-        <v>-0.04270326469418592</v>
+        <v>-0.04270326410547406</v>
       </c>
       <c r="O187" s="2" t="inlineStr">
         <is>
@@ -10410,10 +10410,10 @@
         <v>0</v>
       </c>
       <c r="H188" s="2" t="n">
-        <v>33.707611775792</v>
+        <v>33.70761197084526</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>21.64140312556706</v>
+        <v>21.64140318058951</v>
       </c>
       <c r="J188" s="2" t="n">
         <v>0.6639172934029418</v>
@@ -10428,7 +10428,7 @@
         <v>-1</v>
       </c>
       <c r="N188" s="2" t="n">
-        <v>-3.578158330846406</v>
+        <v>-3.578158333369439</v>
       </c>
       <c r="O188" s="2" t="inlineStr">
         <is>
@@ -10463,10 +10463,10 @@
         <v>0</v>
       </c>
       <c r="H189" s="2" t="n">
-        <v>11.52083645774805</v>
+        <v>11.52083640148439</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>13.87735769352242</v>
+        <v>13.87735777015562</v>
       </c>
       <c r="J189" s="2" t="n">
         <v>0.0007237947524880445</v>
@@ -10481,7 +10481,7 @@
         <v>-1</v>
       </c>
       <c r="N189" s="2" t="n">
-        <v>-1.167508172287577</v>
+        <v>-1.167508172077322</v>
       </c>
       <c r="O189" s="2" t="inlineStr">
         <is>
@@ -10569,10 +10569,10 @@
         <v>0</v>
       </c>
       <c r="H191" s="2" t="n">
-        <v>42.25252714007105</v>
+        <v>42.25252722435907</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>11.90996749165673</v>
+        <v>11.90996773680879</v>
       </c>
       <c r="J191" s="2" t="n">
         <v>0.3479774444421553</v>
@@ -10587,7 +10587,7 @@
         <v>-1</v>
       </c>
       <c r="N191" s="2" t="n">
-        <v>-1.007587810217316</v>
+        <v>-1.007587810413554</v>
       </c>
       <c r="O191" s="2" t="inlineStr">
         <is>
@@ -10675,10 +10675,10 @@
         <v>0</v>
       </c>
       <c r="H193" s="2" t="n">
-        <v>37.64827166962808</v>
+        <v>37.64827185381522</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>18.93759940074638</v>
+        <v>18.93759925756041</v>
       </c>
       <c r="J193" s="2" t="n">
         <v>0.8686707207964138</v>
@@ -10834,10 +10834,10 @@
         <v>0</v>
       </c>
       <c r="H196" s="2" t="n">
-        <v>37.92450674919996</v>
+        <v>37.92450678117308</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>11.06908946212346</v>
+        <v>11.06908942392103</v>
       </c>
       <c r="J196" s="2" t="n">
         <v>1.224654676933049</v>
@@ -10852,7 +10852,7 @@
         <v>-1</v>
       </c>
       <c r="N196" s="2" t="n">
-        <v>-0.04423553574239592</v>
+        <v>-0.04423553577043335</v>
       </c>
       <c r="O196" s="2" t="inlineStr">
         <is>
@@ -10940,10 +10940,10 @@
         <v>0</v>
       </c>
       <c r="H198" s="2" t="n">
-        <v>35.66960352142559</v>
+        <v>35.66960374520947</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>20.96430509292411</v>
+        <v>20.96430506370876</v>
       </c>
       <c r="J198" s="2" t="n">
         <v>0.6803719756736204</v>
@@ -10958,7 +10958,7 @@
         <v>-1</v>
       </c>
       <c r="N198" s="2" t="n">
-        <v>-0.8898085145268805</v>
+        <v>-0.8898085144988355</v>
       </c>
       <c r="O198" s="2" t="inlineStr">
         <is>
@@ -11152,10 +11152,10 @@
         <v>0</v>
       </c>
       <c r="H202" s="2" t="n">
-        <v>40.75437448832061</v>
+        <v>40.75437455872663</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>14.51016831394782</v>
+        <v>14.5101682094784</v>
       </c>
       <c r="J202" s="2" t="n">
         <v>0.899545007484485</v>
@@ -11170,7 +11170,7 @@
         <v>-1</v>
       </c>
       <c r="N202" s="2" t="n">
-        <v>0.003573072225737828</v>
+        <v>0.003573072127620924</v>
       </c>
       <c r="O202" s="2" t="inlineStr">
         <is>
@@ -11191,7 +11191,7 @@
         <v/>
       </c>
       <c r="D203" s="2" t="n">
-        <v>201.8951697132856</v>
+        <v>201.8951697132857</v>
       </c>
       <c r="E203" s="2" t="n">
         <v>27</v>
@@ -11205,10 +11205,10 @@
         <v>0</v>
       </c>
       <c r="H203" s="2" t="n">
-        <v>31.56020229704599</v>
+        <v>31.56020218569969</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>14.93431082612478</v>
+        <v>14.93431083001839</v>
       </c>
       <c r="J203" s="2" t="n">
         <v>0.5035535472288432</v>
@@ -11223,7 +11223,7 @@
         <v>-1</v>
       </c>
       <c r="N203" s="2" t="n">
-        <v>-0.01043953151433041</v>
+        <v>-0.01043953150031429</v>
       </c>
       <c r="O203" s="2" t="inlineStr">
         <is>
@@ -11311,10 +11311,10 @@
         <v>0</v>
       </c>
       <c r="H205" s="2" t="n">
-        <v>36.0237349429537</v>
+        <v>36.02373385377551</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>10.45211785658284</v>
+        <v>10.45211772143344</v>
       </c>
       <c r="J205" s="2" t="n">
         <v>0.8388056787664476</v>
@@ -11329,7 +11329,7 @@
         <v>-1</v>
       </c>
       <c r="N205" s="2" t="n">
-        <v>-0.005477318234435813</v>
+        <v>-0.005477317982130636</v>
       </c>
       <c r="O205" s="2" t="inlineStr">
         <is>
@@ -11470,10 +11470,10 @@
         <v>0</v>
       </c>
       <c r="H208" s="2" t="n">
-        <v>37.17449661356735</v>
+        <v>37.17449665533236</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>13.76474790888678</v>
+        <v>13.76474785115363</v>
       </c>
       <c r="J208" s="2" t="n">
         <v>7.068907809215692</v>
@@ -11488,7 +11488,7 @@
         <v>-1</v>
       </c>
       <c r="N208" s="2" t="n">
-        <v>0.00850697946763368</v>
+        <v>0.008506979448010737</v>
       </c>
       <c r="O208" s="2" t="inlineStr">
         <is>
@@ -11509,7 +11509,7 @@
         <v/>
       </c>
       <c r="D209" s="2" t="n">
-        <v>188.548744267579</v>
+        <v>188.5487442675791</v>
       </c>
       <c r="E209" s="2" t="n">
         <v>83.5</v>
@@ -11523,10 +11523,10 @@
         <v>0</v>
       </c>
       <c r="H209" s="2" t="n">
-        <v>41.43273631009949</v>
+        <v>41.43273639896044</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>31.47796784498475</v>
+        <v>31.47796778492597</v>
       </c>
       <c r="J209" s="2" t="n">
         <v>0.2762989598312651</v>
@@ -11541,7 +11541,7 @@
         <v>-1</v>
       </c>
       <c r="N209" s="2" t="n">
-        <v>-0.9909846641040378</v>
+        <v>-0.9909846643563416</v>
       </c>
       <c r="O209" s="2" t="inlineStr">
         <is>
@@ -11562,7 +11562,7 @@
         <v/>
       </c>
       <c r="D210" s="2" t="n">
-        <v>186.3929909916752</v>
+        <v>186.3929909916751</v>
       </c>
       <c r="E210" s="2" t="n">
         <v>17.45</v>
@@ -11576,10 +11576,10 @@
         <v>0</v>
       </c>
       <c r="H210" s="2" t="n">
-        <v>24.9008997119485</v>
+        <v>24.90089979955948</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>10.18580612455647</v>
+        <v>10.18580616809307</v>
       </c>
       <c r="J210" s="2" t="n">
         <v>1.092880909115284</v>
@@ -11594,7 +11594,7 @@
         <v>-1</v>
       </c>
       <c r="N210" s="2" t="n">
-        <v>-0.1672196176607952</v>
+        <v>-0.1672196176888292</v>
       </c>
       <c r="O210" s="2" t="inlineStr">
         <is>
@@ -11682,10 +11682,10 @@
         <v>0</v>
       </c>
       <c r="H212" s="2" t="n">
-        <v>26.12179455485359</v>
+        <v>26.12179460758146</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>22.37968355597135</v>
+        <v>22.37968361476535</v>
       </c>
       <c r="J212" s="2" t="n">
         <v>0.3800663333953394</v>
@@ -11700,7 +11700,7 @@
         <v>-1</v>
       </c>
       <c r="N212" s="2" t="n">
-        <v>-0.2879941181293874</v>
+        <v>-0.2879941181994723</v>
       </c>
       <c r="O212" s="2" t="inlineStr">
         <is>
@@ -11788,10 +11788,10 @@
         <v>0</v>
       </c>
       <c r="H214" s="2" t="n">
-        <v>26.09631034049298</v>
+        <v>26.09631005198662</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>20.96952813684501</v>
+        <v>20.96952858809449</v>
       </c>
       <c r="J214" s="2" t="n">
         <v>0.701392221277404</v>
@@ -11806,7 +11806,7 @@
         <v>-1</v>
       </c>
       <c r="N214" s="2" t="n">
-        <v>-0.2645548769745709</v>
+        <v>-0.2645548761475687</v>
       </c>
       <c r="O214" s="2" t="inlineStr">
         <is>
@@ -11841,10 +11841,10 @@
         <v>0</v>
       </c>
       <c r="H215" s="2" t="n">
-        <v>30.55866308095929</v>
+        <v>30.55866305749589</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>18.80052288499933</v>
+        <v>18.80052296452055</v>
       </c>
       <c r="J215" s="2" t="n">
         <v>0.6164791211884133</v>
@@ -11859,7 +11859,7 @@
         <v>-1</v>
       </c>
       <c r="N215" s="2" t="n">
-        <v>-4.909249971848601</v>
+        <v>-4.909249971680375</v>
       </c>
       <c r="O215" s="2" t="inlineStr">
         <is>
@@ -11947,10 +11947,10 @@
         <v>0</v>
       </c>
       <c r="H217" s="2" t="n">
-        <v>30.461679581916</v>
+        <v>30.46167958723071</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>17.52097940179847</v>
+        <v>17.52097942663049</v>
       </c>
       <c r="J217" s="2" t="n">
         <v>0.8883898913240174</v>
@@ -12000,10 +12000,10 @@
         <v>0</v>
       </c>
       <c r="H218" s="2" t="n">
-        <v>37.23514730692923</v>
+        <v>37.23514732820649</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>12.36999375487721</v>
+        <v>12.36999376717008</v>
       </c>
       <c r="J218" s="2" t="n">
         <v>0.8601649755493119</v>
@@ -12106,10 +12106,10 @@
         <v>0</v>
       </c>
       <c r="H220" s="2" t="n">
-        <v>45.03735723515509</v>
+        <v>45.0373579518564</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>16.42150005486003</v>
+        <v>16.42150015051694</v>
       </c>
       <c r="J220" s="2" t="n">
         <v>0.6020460670612601</v>
@@ -12124,7 +12124,7 @@
         <v>-1</v>
       </c>
       <c r="N220" s="2" t="n">
-        <v>-0.480209510424734</v>
+        <v>-0.4802095105649107</v>
       </c>
       <c r="O220" s="2" t="inlineStr">
         <is>
@@ -12198,7 +12198,7 @@
         <v/>
       </c>
       <c r="D222" s="2" t="n">
-        <v>152.3936047930341</v>
+        <v>152.3936047930342</v>
       </c>
       <c r="E222" s="2" t="n">
         <v>707</v>
@@ -12212,10 +12212,10 @@
         <v>0</v>
       </c>
       <c r="H222" s="2" t="n">
-        <v>39.47981492870313</v>
+        <v>39.47981506622715</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>15.59870959992594</v>
+        <v>15.5987095748841</v>
       </c>
       <c r="J222" s="2" t="n">
         <v>0.6015291717014272</v>
@@ -12230,7 +12230,7 @@
         <v>-1</v>
       </c>
       <c r="N222" s="2" t="n">
-        <v>-4.162707538478815</v>
+        <v>-4.162707543524883</v>
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
@@ -12424,10 +12424,10 @@
         <v>0</v>
       </c>
       <c r="H226" s="2" t="n">
-        <v>33.0493700665655</v>
+        <v>33.04937016307447</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>12.02310443653079</v>
+        <v>12.02310433433937</v>
       </c>
       <c r="J226" s="2" t="n">
         <v>0.728202929940001</v>
@@ -12442,7 +12442,7 @@
         <v>-1</v>
       </c>
       <c r="N226" s="2" t="n">
-        <v>-4.521223237820407</v>
+        <v>-4.521223238941801</v>
       </c>
       <c r="O226" s="2" t="inlineStr">
         <is>
@@ -12530,10 +12530,10 @@
         <v>0</v>
       </c>
       <c r="H228" s="2" t="n">
-        <v>21.99524606877875</v>
+        <v>21.99524675980352</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>27.79513796071957</v>
+        <v>27.79513805640714</v>
       </c>
       <c r="J228" s="2" t="n">
         <v>1.12843448229242</v>
@@ -12548,7 +12548,7 @@
         <v>-1</v>
       </c>
       <c r="N228" s="2" t="n">
-        <v>-1.012220413721808</v>
+        <v>-1.01222041386198</v>
       </c>
       <c r="O228" s="2" t="inlineStr">
         <is>
@@ -12569,7 +12569,7 @@
         <v/>
       </c>
       <c r="D229" s="2" t="n">
-        <v>127.8823502790383</v>
+        <v>127.8823502790391</v>
       </c>
       <c r="E229" s="2" t="n">
         <v>35.55</v>
@@ -12583,10 +12583,10 @@
         <v>0</v>
       </c>
       <c r="H229" s="2" t="n">
-        <v>31.71083871130759</v>
+        <v>31.71083908503739</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>20.70737139166161</v>
+        <v>20.70737142241301</v>
       </c>
       <c r="J229" s="2" t="n">
         <v>0.7590208083519627</v>
@@ -12601,7 +12601,7 @@
         <v>-1</v>
       </c>
       <c r="N229" s="2" t="n">
-        <v>-0.2216749514324168</v>
+        <v>-0.2216749521052268</v>
       </c>
       <c r="O229" s="2" t="inlineStr">
         <is>
@@ -12636,10 +12636,10 @@
         <v>0</v>
       </c>
       <c r="H230" s="2" t="n">
-        <v>39.35846387667224</v>
+        <v>39.35846373940834</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>10.18354431393332</v>
+        <v>10.18354432118574</v>
       </c>
       <c r="J230" s="2" t="n">
         <v>0.7808789032972285</v>
@@ -12654,7 +12654,7 @@
         <v>-1</v>
       </c>
       <c r="N230" s="2" t="n">
-        <v>-0.1257731960545186</v>
+        <v>-0.1257731958022121</v>
       </c>
       <c r="O230" s="2" t="inlineStr">
         <is>
@@ -12728,7 +12728,7 @@
         <v/>
       </c>
       <c r="D232" s="2" t="n">
-        <v>110.5586899048245</v>
+        <v>110.5586899048243</v>
       </c>
       <c r="E232" s="2" t="n">
         <v>22.2</v>
@@ -12742,10 +12742,10 @@
         <v>0</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>41.8151434594628</v>
+        <v>41.81514344021141</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>9.98325805571517</v>
+        <v>9.983258091058866</v>
       </c>
       <c r="J232" s="2" t="n">
         <v>0.4883685917389942</v>
@@ -12760,7 +12760,7 @@
         <v>-1</v>
       </c>
       <c r="N232" s="2" t="n">
-        <v>-0.006643671489805103</v>
+        <v>-0.006643671503821919</v>
       </c>
       <c r="O232" s="2" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         <v/>
       </c>
       <c r="D233" s="2" t="n">
-        <v>109.3628552811357</v>
+        <v>109.3628552811311</v>
       </c>
       <c r="E233" s="2" t="n">
         <v>270</v>
@@ -12795,10 +12795,10 @@
         <v>0</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>29.17258957576664</v>
+        <v>29.17259030138057</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>14.04848098066682</v>
+        <v>14.04848104614486</v>
       </c>
       <c r="J233" s="2" t="n">
         <v>0.9626515930409731</v>
@@ -12813,7 +12813,7 @@
         <v>-1</v>
       </c>
       <c r="N233" s="2" t="n">
-        <v>-1.839017701657149</v>
+        <v>-1.83901770922635</v>
       </c>
       <c r="O233" s="2" t="inlineStr">
         <is>
@@ -12834,7 +12834,7 @@
         <v/>
       </c>
       <c r="D234" s="2" t="n">
-        <v>109.1527221376194</v>
+        <v>109.1527221376195</v>
       </c>
       <c r="E234" s="2" t="n">
         <v>35.4</v>
@@ -12848,10 +12848,10 @@
         <v>0</v>
       </c>
       <c r="H234" s="2" t="n">
-        <v>27.32345356241872</v>
+        <v>27.32345349500625</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>15.78256059290033</v>
+        <v>15.78256061732305</v>
       </c>
       <c r="J234" s="2" t="n">
         <v>1.651589340605032</v>
@@ -12866,7 +12866,7 @@
         <v>-1</v>
       </c>
       <c r="N234" s="2" t="n">
-        <v>-0.1539173754219456</v>
+        <v>-0.153917375379898</v>
       </c>
       <c r="O234" s="2" t="inlineStr">
         <is>
@@ -13007,10 +13007,10 @@
         <v>0</v>
       </c>
       <c r="H237" s="2" t="n">
-        <v>32.99529531099292</v>
+        <v>32.99529561731219</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>19.23361674416959</v>
+        <v>19.23361670760579</v>
       </c>
       <c r="J237" s="2" t="n">
         <v>0.760399565868991</v>
@@ -13025,7 +13025,7 @@
         <v>-1</v>
       </c>
       <c r="N237" s="2" t="n">
-        <v>0.01899602823783691</v>
+        <v>0.01899602827988706</v>
       </c>
       <c r="O237" s="2" t="inlineStr">
         <is>

</xml_diff>